<commit_message>
Update NGO dashboard layout with active requirements list, navigate controls, and restricted categories on mobile
</commit_message>
<xml_diff>
--- a/e2e-tests/reports/test-report.xlsx
+++ b/e2e-tests/reports/test-report.xlsx
@@ -42,19 +42,19 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>17.27s</t>
+    <t>17.19s</t>
   </si>
   <si>
     <t>Average Test Duration</t>
   </si>
   <si>
-    <t>34.55ms</t>
+    <t>34.37ms</t>
   </si>
   <si>
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>7/23/2026, 2:30:55 PM</t>
+    <t>7/23/2026, 3:23:00 PM</t>
   </si>
   <si>
     <t>Category</t>
@@ -3684,7 +3684,7 @@
         <v>100</v>
       </c>
       <c r="G2">
-        <v>35.6</v>
+        <v>34.46</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3707,7 +3707,7 @@
         <v>100</v>
       </c>
       <c r="G3">
-        <v>32.66</v>
+        <v>34.24</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3730,7 +3730,7 @@
         <v>100</v>
       </c>
       <c r="G4">
-        <v>35.04</v>
+        <v>35.46</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3753,7 +3753,7 @@
         <v>100</v>
       </c>
       <c r="G5">
-        <v>34.24</v>
+        <v>33.54</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -3776,7 +3776,7 @@
         <v>100</v>
       </c>
       <c r="G6">
-        <v>36.94</v>
+        <v>36.26</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -3799,7 +3799,7 @@
         <v>100</v>
       </c>
       <c r="G7">
-        <v>35.1</v>
+        <v>33.88</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -3822,7 +3822,7 @@
         <v>100</v>
       </c>
       <c r="G8">
-        <v>32</v>
+        <v>34.64</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3845,7 +3845,7 @@
         <v>100</v>
       </c>
       <c r="G9">
-        <v>34.78</v>
+        <v>31.58</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3868,7 +3868,7 @@
         <v>100</v>
       </c>
       <c r="G10">
-        <v>35.46</v>
+        <v>33.64</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3891,7 +3891,7 @@
         <v>100</v>
       </c>
       <c r="G11">
-        <v>33.64</v>
+        <v>36.04</v>
       </c>
     </row>
   </sheetData>
@@ -3957,7 +3957,7 @@
         <v>37</v>
       </c>
       <c r="F2">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G2" t="s">
         <v>38</v>
@@ -3983,7 +3983,7 @@
         <v>37</v>
       </c>
       <c r="F3">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="G3" t="s">
         <v>38</v>
@@ -4035,7 +4035,7 @@
         <v>37</v>
       </c>
       <c r="F5">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G5" t="s">
         <v>38</v>
@@ -4061,7 +4061,7 @@
         <v>37</v>
       </c>
       <c r="F6">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G6" t="s">
         <v>38</v>
@@ -4139,7 +4139,7 @@
         <v>37</v>
       </c>
       <c r="F9">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
         <v>38</v>
@@ -4191,7 +4191,7 @@
         <v>37</v>
       </c>
       <c r="F11">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="G11" t="s">
         <v>38</v>
@@ -4217,7 +4217,7 @@
         <v>37</v>
       </c>
       <c r="F12">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="G12" t="s">
         <v>38</v>
@@ -4243,7 +4243,7 @@
         <v>37</v>
       </c>
       <c r="F13">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="G13" t="s">
         <v>38</v>
@@ -4269,7 +4269,7 @@
         <v>37</v>
       </c>
       <c r="F14">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="G14" t="s">
         <v>38</v>
@@ -4295,7 +4295,7 @@
         <v>37</v>
       </c>
       <c r="F15">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="G15" t="s">
         <v>38</v>
@@ -4321,7 +4321,7 @@
         <v>37</v>
       </c>
       <c r="F16">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="G16" t="s">
         <v>38</v>
@@ -4347,7 +4347,7 @@
         <v>37</v>
       </c>
       <c r="F17">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="G17" t="s">
         <v>38</v>
@@ -4373,7 +4373,7 @@
         <v>37</v>
       </c>
       <c r="F18">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="G18" t="s">
         <v>38</v>
@@ -4399,7 +4399,7 @@
         <v>37</v>
       </c>
       <c r="F19">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G19" t="s">
         <v>38</v>
@@ -4425,7 +4425,7 @@
         <v>37</v>
       </c>
       <c r="F20">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="G20" t="s">
         <v>38</v>
@@ -4451,7 +4451,7 @@
         <v>37</v>
       </c>
       <c r="F21">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="G21" t="s">
         <v>38</v>
@@ -4503,7 +4503,7 @@
         <v>37</v>
       </c>
       <c r="F23">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G23" t="s">
         <v>38</v>
@@ -4529,7 +4529,7 @@
         <v>37</v>
       </c>
       <c r="F24">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="G24" t="s">
         <v>38</v>
@@ -4555,7 +4555,7 @@
         <v>37</v>
       </c>
       <c r="F25">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="G25" t="s">
         <v>38</v>
@@ -4581,7 +4581,7 @@
         <v>37</v>
       </c>
       <c r="F26">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="G26" t="s">
         <v>38</v>
@@ -4607,7 +4607,7 @@
         <v>37</v>
       </c>
       <c r="F27">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G27" t="s">
         <v>38</v>
@@ -4633,7 +4633,7 @@
         <v>37</v>
       </c>
       <c r="F28">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="G28" t="s">
         <v>38</v>
@@ -4659,7 +4659,7 @@
         <v>37</v>
       </c>
       <c r="F29">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="G29" t="s">
         <v>38</v>
@@ -4685,7 +4685,7 @@
         <v>37</v>
       </c>
       <c r="F30">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="G30" t="s">
         <v>38</v>
@@ -4711,7 +4711,7 @@
         <v>37</v>
       </c>
       <c r="F31">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="G31" t="s">
         <v>38</v>
@@ -4737,7 +4737,7 @@
         <v>37</v>
       </c>
       <c r="F32">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G32" t="s">
         <v>38</v>
@@ -4763,7 +4763,7 @@
         <v>37</v>
       </c>
       <c r="F33">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="G33" t="s">
         <v>38</v>
@@ -4789,7 +4789,7 @@
         <v>37</v>
       </c>
       <c r="F34">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G34" t="s">
         <v>38</v>
@@ -4815,7 +4815,7 @@
         <v>37</v>
       </c>
       <c r="F35">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G35" t="s">
         <v>38</v>
@@ -4841,7 +4841,7 @@
         <v>37</v>
       </c>
       <c r="F36">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="G36" t="s">
         <v>38</v>
@@ -4867,7 +4867,7 @@
         <v>37</v>
       </c>
       <c r="F37">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="G37" t="s">
         <v>38</v>
@@ -4893,7 +4893,7 @@
         <v>37</v>
       </c>
       <c r="F38">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="G38" t="s">
         <v>38</v>
@@ -4919,7 +4919,7 @@
         <v>37</v>
       </c>
       <c r="F39">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="G39" t="s">
         <v>38</v>
@@ -4945,7 +4945,7 @@
         <v>37</v>
       </c>
       <c r="F40">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="G40" t="s">
         <v>38</v>
@@ -4971,7 +4971,7 @@
         <v>37</v>
       </c>
       <c r="F41">
-        <v>49</v>
+        <v>26</v>
       </c>
       <c r="G41" t="s">
         <v>38</v>
@@ -4997,7 +4997,7 @@
         <v>37</v>
       </c>
       <c r="F42">
-        <v>25</v>
+        <v>50</v>
       </c>
       <c r="G42" t="s">
         <v>38</v>
@@ -5023,7 +5023,7 @@
         <v>37</v>
       </c>
       <c r="F43">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="G43" t="s">
         <v>38</v>
@@ -5049,7 +5049,7 @@
         <v>37</v>
       </c>
       <c r="F44">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="G44" t="s">
         <v>38</v>
@@ -5075,7 +5075,7 @@
         <v>37</v>
       </c>
       <c r="F45">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G45" t="s">
         <v>38</v>
@@ -5101,7 +5101,7 @@
         <v>37</v>
       </c>
       <c r="F46">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="G46" t="s">
         <v>38</v>
@@ -5127,7 +5127,7 @@
         <v>37</v>
       </c>
       <c r="F47">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G47" t="s">
         <v>38</v>
@@ -5153,7 +5153,7 @@
         <v>37</v>
       </c>
       <c r="F48">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G48" t="s">
         <v>38</v>
@@ -5179,7 +5179,7 @@
         <v>37</v>
       </c>
       <c r="F49">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="G49" t="s">
         <v>38</v>
@@ -5205,7 +5205,7 @@
         <v>37</v>
       </c>
       <c r="F50">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G50" t="s">
         <v>38</v>
@@ -5231,7 +5231,7 @@
         <v>37</v>
       </c>
       <c r="F51">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G51" t="s">
         <v>38</v>
@@ -5257,7 +5257,7 @@
         <v>37</v>
       </c>
       <c r="F52">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G52" t="s">
         <v>38</v>
@@ -5283,7 +5283,7 @@
         <v>37</v>
       </c>
       <c r="F53">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G53" t="s">
         <v>38</v>
@@ -5309,7 +5309,7 @@
         <v>37</v>
       </c>
       <c r="F54">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="G54" t="s">
         <v>38</v>
@@ -5335,7 +5335,7 @@
         <v>37</v>
       </c>
       <c r="F55">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="G55" t="s">
         <v>38</v>
@@ -5361,7 +5361,7 @@
         <v>37</v>
       </c>
       <c r="F56">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G56" t="s">
         <v>38</v>
@@ -5387,7 +5387,7 @@
         <v>37</v>
       </c>
       <c r="F57">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="G57" t="s">
         <v>38</v>
@@ -5413,7 +5413,7 @@
         <v>37</v>
       </c>
       <c r="F58">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G58" t="s">
         <v>38</v>
@@ -5439,7 +5439,7 @@
         <v>37</v>
       </c>
       <c r="F59">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G59" t="s">
         <v>38</v>
@@ -5465,7 +5465,7 @@
         <v>37</v>
       </c>
       <c r="F60">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G60" t="s">
         <v>38</v>
@@ -5491,7 +5491,7 @@
         <v>37</v>
       </c>
       <c r="F61">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="G61" t="s">
         <v>38</v>
@@ -5517,7 +5517,7 @@
         <v>37</v>
       </c>
       <c r="F62">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G62" t="s">
         <v>38</v>
@@ -5543,7 +5543,7 @@
         <v>37</v>
       </c>
       <c r="F63">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="G63" t="s">
         <v>38</v>
@@ -5569,7 +5569,7 @@
         <v>37</v>
       </c>
       <c r="F64">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="G64" t="s">
         <v>38</v>
@@ -5595,7 +5595,7 @@
         <v>37</v>
       </c>
       <c r="F65">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G65" t="s">
         <v>38</v>
@@ -5621,7 +5621,7 @@
         <v>37</v>
       </c>
       <c r="F66">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="G66" t="s">
         <v>38</v>
@@ -5647,7 +5647,7 @@
         <v>37</v>
       </c>
       <c r="F67">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G67" t="s">
         <v>38</v>
@@ -5673,7 +5673,7 @@
         <v>37</v>
       </c>
       <c r="F68">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G68" t="s">
         <v>38</v>
@@ -5699,7 +5699,7 @@
         <v>37</v>
       </c>
       <c r="F69">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G69" t="s">
         <v>38</v>
@@ -5725,7 +5725,7 @@
         <v>37</v>
       </c>
       <c r="F70">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G70" t="s">
         <v>38</v>
@@ -5751,7 +5751,7 @@
         <v>37</v>
       </c>
       <c r="F71">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="G71" t="s">
         <v>38</v>
@@ -5777,7 +5777,7 @@
         <v>37</v>
       </c>
       <c r="F72">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G72" t="s">
         <v>38</v>
@@ -5803,7 +5803,7 @@
         <v>37</v>
       </c>
       <c r="F73">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="G73" t="s">
         <v>38</v>
@@ -5829,7 +5829,7 @@
         <v>37</v>
       </c>
       <c r="F74">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="G74" t="s">
         <v>38</v>
@@ -5855,7 +5855,7 @@
         <v>37</v>
       </c>
       <c r="F75">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G75" t="s">
         <v>38</v>
@@ -5881,7 +5881,7 @@
         <v>37</v>
       </c>
       <c r="F76">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="G76" t="s">
         <v>38</v>
@@ -5907,7 +5907,7 @@
         <v>37</v>
       </c>
       <c r="F77">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G77" t="s">
         <v>38</v>
@@ -5933,7 +5933,7 @@
         <v>37</v>
       </c>
       <c r="F78">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G78" t="s">
         <v>38</v>
@@ -5959,7 +5959,7 @@
         <v>37</v>
       </c>
       <c r="F79">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="G79" t="s">
         <v>38</v>
@@ -5985,7 +5985,7 @@
         <v>37</v>
       </c>
       <c r="F80">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G80" t="s">
         <v>38</v>
@@ -6011,7 +6011,7 @@
         <v>37</v>
       </c>
       <c r="F81">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="G81" t="s">
         <v>38</v>
@@ -6037,7 +6037,7 @@
         <v>37</v>
       </c>
       <c r="F82">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="G82" t="s">
         <v>38</v>
@@ -6063,7 +6063,7 @@
         <v>37</v>
       </c>
       <c r="F83">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G83" t="s">
         <v>38</v>
@@ -6089,7 +6089,7 @@
         <v>37</v>
       </c>
       <c r="F84">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="G84" t="s">
         <v>38</v>
@@ -6115,7 +6115,7 @@
         <v>37</v>
       </c>
       <c r="F85">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="G85" t="s">
         <v>38</v>
@@ -6141,7 +6141,7 @@
         <v>37</v>
       </c>
       <c r="F86">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G86" t="s">
         <v>38</v>
@@ -6193,7 +6193,7 @@
         <v>37</v>
       </c>
       <c r="F88">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G88" t="s">
         <v>38</v>
@@ -6219,7 +6219,7 @@
         <v>37</v>
       </c>
       <c r="F89">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G89" t="s">
         <v>38</v>
@@ -6245,7 +6245,7 @@
         <v>37</v>
       </c>
       <c r="F90">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="G90" t="s">
         <v>38</v>
@@ -6271,7 +6271,7 @@
         <v>37</v>
       </c>
       <c r="F91">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="G91" t="s">
         <v>38</v>
@@ -6297,7 +6297,7 @@
         <v>37</v>
       </c>
       <c r="F92">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="G92" t="s">
         <v>38</v>
@@ -6323,7 +6323,7 @@
         <v>37</v>
       </c>
       <c r="F93">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="G93" t="s">
         <v>38</v>
@@ -6349,7 +6349,7 @@
         <v>37</v>
       </c>
       <c r="F94">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G94" t="s">
         <v>38</v>
@@ -6375,7 +6375,7 @@
         <v>37</v>
       </c>
       <c r="F95">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="G95" t="s">
         <v>38</v>
@@ -6401,7 +6401,7 @@
         <v>37</v>
       </c>
       <c r="F96">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="G96" t="s">
         <v>38</v>
@@ -6427,7 +6427,7 @@
         <v>37</v>
       </c>
       <c r="F97">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G97" t="s">
         <v>38</v>
@@ -6453,7 +6453,7 @@
         <v>37</v>
       </c>
       <c r="F98">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G98" t="s">
         <v>38</v>
@@ -6479,7 +6479,7 @@
         <v>37</v>
       </c>
       <c r="F99">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G99" t="s">
         <v>38</v>
@@ -6505,7 +6505,7 @@
         <v>37</v>
       </c>
       <c r="F100">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="G100" t="s">
         <v>38</v>
@@ -6531,7 +6531,7 @@
         <v>37</v>
       </c>
       <c r="F101">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="G101" t="s">
         <v>38</v>
@@ -6557,7 +6557,7 @@
         <v>37</v>
       </c>
       <c r="F102">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G102" t="s">
         <v>38</v>
@@ -6583,7 +6583,7 @@
         <v>37</v>
       </c>
       <c r="F103">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="G103" t="s">
         <v>38</v>
@@ -6609,7 +6609,7 @@
         <v>37</v>
       </c>
       <c r="F104">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="G104" t="s">
         <v>38</v>
@@ -6635,7 +6635,7 @@
         <v>37</v>
       </c>
       <c r="F105">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="G105" t="s">
         <v>38</v>
@@ -6661,7 +6661,7 @@
         <v>37</v>
       </c>
       <c r="F106">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G106" t="s">
         <v>38</v>
@@ -6687,7 +6687,7 @@
         <v>37</v>
       </c>
       <c r="F107">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="G107" t="s">
         <v>38</v>
@@ -6713,7 +6713,7 @@
         <v>37</v>
       </c>
       <c r="F108">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="G108" t="s">
         <v>38</v>
@@ -6739,7 +6739,7 @@
         <v>37</v>
       </c>
       <c r="F109">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="G109" t="s">
         <v>38</v>
@@ -6765,7 +6765,7 @@
         <v>37</v>
       </c>
       <c r="F110">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="G110" t="s">
         <v>38</v>
@@ -6791,7 +6791,7 @@
         <v>37</v>
       </c>
       <c r="F111">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="G111" t="s">
         <v>38</v>
@@ -6817,7 +6817,7 @@
         <v>37</v>
       </c>
       <c r="F112">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G112" t="s">
         <v>38</v>
@@ -6843,7 +6843,7 @@
         <v>37</v>
       </c>
       <c r="F113">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="G113" t="s">
         <v>38</v>
@@ -6869,7 +6869,7 @@
         <v>37</v>
       </c>
       <c r="F114">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="G114" t="s">
         <v>38</v>
@@ -6895,7 +6895,7 @@
         <v>37</v>
       </c>
       <c r="F115">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G115" t="s">
         <v>38</v>
@@ -6921,7 +6921,7 @@
         <v>37</v>
       </c>
       <c r="F116">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="G116" t="s">
         <v>38</v>
@@ -6947,7 +6947,7 @@
         <v>37</v>
       </c>
       <c r="F117">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="G117" t="s">
         <v>38</v>
@@ -6973,7 +6973,7 @@
         <v>37</v>
       </c>
       <c r="F118">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G118" t="s">
         <v>38</v>
@@ -6999,7 +6999,7 @@
         <v>37</v>
       </c>
       <c r="F119">
-        <v>47</v>
+        <v>31</v>
       </c>
       <c r="G119" t="s">
         <v>38</v>
@@ -7025,7 +7025,7 @@
         <v>37</v>
       </c>
       <c r="F120">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="G120" t="s">
         <v>38</v>
@@ -7051,7 +7051,7 @@
         <v>37</v>
       </c>
       <c r="F121">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="G121" t="s">
         <v>38</v>
@@ -7077,7 +7077,7 @@
         <v>37</v>
       </c>
       <c r="F122">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="G122" t="s">
         <v>38</v>
@@ -7129,7 +7129,7 @@
         <v>37</v>
       </c>
       <c r="F124">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G124" t="s">
         <v>38</v>
@@ -7155,7 +7155,7 @@
         <v>37</v>
       </c>
       <c r="F125">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G125" t="s">
         <v>38</v>
@@ -7181,7 +7181,7 @@
         <v>37</v>
       </c>
       <c r="F126">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="G126" t="s">
         <v>38</v>
@@ -7207,7 +7207,7 @@
         <v>37</v>
       </c>
       <c r="F127">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G127" t="s">
         <v>38</v>
@@ -7233,7 +7233,7 @@
         <v>37</v>
       </c>
       <c r="F128">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="G128" t="s">
         <v>38</v>
@@ -7259,7 +7259,7 @@
         <v>37</v>
       </c>
       <c r="F129">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G129" t="s">
         <v>38</v>
@@ -7285,7 +7285,7 @@
         <v>37</v>
       </c>
       <c r="F130">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="G130" t="s">
         <v>38</v>
@@ -7311,7 +7311,7 @@
         <v>37</v>
       </c>
       <c r="F131">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="G131" t="s">
         <v>38</v>
@@ -7337,7 +7337,7 @@
         <v>37</v>
       </c>
       <c r="F132">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="G132" t="s">
         <v>38</v>
@@ -7363,7 +7363,7 @@
         <v>37</v>
       </c>
       <c r="F133">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="G133" t="s">
         <v>38</v>
@@ -7389,7 +7389,7 @@
         <v>37</v>
       </c>
       <c r="F134">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="G134" t="s">
         <v>38</v>
@@ -7415,7 +7415,7 @@
         <v>37</v>
       </c>
       <c r="F135">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="G135" t="s">
         <v>38</v>
@@ -7441,7 +7441,7 @@
         <v>37</v>
       </c>
       <c r="F136">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="G136" t="s">
         <v>38</v>
@@ -7467,7 +7467,7 @@
         <v>37</v>
       </c>
       <c r="F137">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="G137" t="s">
         <v>38</v>
@@ -7493,7 +7493,7 @@
         <v>37</v>
       </c>
       <c r="F138">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="G138" t="s">
         <v>38</v>
@@ -7519,7 +7519,7 @@
         <v>37</v>
       </c>
       <c r="F139">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="G139" t="s">
         <v>38</v>
@@ -7545,7 +7545,7 @@
         <v>37</v>
       </c>
       <c r="F140">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="G140" t="s">
         <v>38</v>
@@ -7571,7 +7571,7 @@
         <v>37</v>
       </c>
       <c r="F141">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G141" t="s">
         <v>38</v>
@@ -7597,7 +7597,7 @@
         <v>37</v>
       </c>
       <c r="F142">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="G142" t="s">
         <v>38</v>
@@ -7623,7 +7623,7 @@
         <v>37</v>
       </c>
       <c r="F143">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G143" t="s">
         <v>38</v>
@@ -7649,7 +7649,7 @@
         <v>37</v>
       </c>
       <c r="F144">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="G144" t="s">
         <v>38</v>
@@ -7675,7 +7675,7 @@
         <v>37</v>
       </c>
       <c r="F145">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="G145" t="s">
         <v>38</v>
@@ -7701,7 +7701,7 @@
         <v>37</v>
       </c>
       <c r="F146">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G146" t="s">
         <v>38</v>
@@ -7727,7 +7727,7 @@
         <v>37</v>
       </c>
       <c r="F147">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G147" t="s">
         <v>38</v>
@@ -7753,7 +7753,7 @@
         <v>37</v>
       </c>
       <c r="F148">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="G148" t="s">
         <v>38</v>
@@ -7779,7 +7779,7 @@
         <v>37</v>
       </c>
       <c r="F149">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="G149" t="s">
         <v>38</v>
@@ -7805,7 +7805,7 @@
         <v>37</v>
       </c>
       <c r="F150">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="G150" t="s">
         <v>38</v>
@@ -7831,7 +7831,7 @@
         <v>37</v>
       </c>
       <c r="F151">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="G151" t="s">
         <v>38</v>
@@ -7857,7 +7857,7 @@
         <v>37</v>
       </c>
       <c r="F152">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G152" t="s">
         <v>38</v>
@@ -7883,7 +7883,7 @@
         <v>37</v>
       </c>
       <c r="F153">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="G153" t="s">
         <v>38</v>
@@ -7909,7 +7909,7 @@
         <v>37</v>
       </c>
       <c r="F154">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G154" t="s">
         <v>38</v>
@@ -7935,7 +7935,7 @@
         <v>37</v>
       </c>
       <c r="F155">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="G155" t="s">
         <v>38</v>
@@ -7961,7 +7961,7 @@
         <v>37</v>
       </c>
       <c r="F156">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="G156" t="s">
         <v>38</v>
@@ -8039,7 +8039,7 @@
         <v>37</v>
       </c>
       <c r="F159">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="G159" t="s">
         <v>38</v>
@@ -8065,7 +8065,7 @@
         <v>37</v>
       </c>
       <c r="F160">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G160" t="s">
         <v>38</v>
@@ -8091,7 +8091,7 @@
         <v>37</v>
       </c>
       <c r="F161">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G161" t="s">
         <v>38</v>
@@ -8117,7 +8117,7 @@
         <v>37</v>
       </c>
       <c r="F162">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="G162" t="s">
         <v>38</v>
@@ -8143,7 +8143,7 @@
         <v>37</v>
       </c>
       <c r="F163">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G163" t="s">
         <v>38</v>
@@ -8169,7 +8169,7 @@
         <v>37</v>
       </c>
       <c r="F164">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="G164" t="s">
         <v>38</v>
@@ -8195,7 +8195,7 @@
         <v>37</v>
       </c>
       <c r="F165">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G165" t="s">
         <v>38</v>
@@ -8221,7 +8221,7 @@
         <v>37</v>
       </c>
       <c r="F166">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="G166" t="s">
         <v>38</v>
@@ -8247,7 +8247,7 @@
         <v>37</v>
       </c>
       <c r="F167">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G167" t="s">
         <v>38</v>
@@ -8273,7 +8273,7 @@
         <v>37</v>
       </c>
       <c r="F168">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G168" t="s">
         <v>38</v>
@@ -8299,7 +8299,7 @@
         <v>37</v>
       </c>
       <c r="F169">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G169" t="s">
         <v>38</v>
@@ -8325,7 +8325,7 @@
         <v>37</v>
       </c>
       <c r="F170">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G170" t="s">
         <v>38</v>
@@ -8351,7 +8351,7 @@
         <v>37</v>
       </c>
       <c r="F171">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="G171" t="s">
         <v>38</v>
@@ -8377,7 +8377,7 @@
         <v>37</v>
       </c>
       <c r="F172">
-        <v>28</v>
+        <v>50</v>
       </c>
       <c r="G172" t="s">
         <v>38</v>
@@ -8403,7 +8403,7 @@
         <v>37</v>
       </c>
       <c r="F173">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="G173" t="s">
         <v>38</v>
@@ -8429,7 +8429,7 @@
         <v>37</v>
       </c>
       <c r="F174">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G174" t="s">
         <v>38</v>
@@ -8455,7 +8455,7 @@
         <v>37</v>
       </c>
       <c r="F175">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G175" t="s">
         <v>38</v>
@@ -8481,7 +8481,7 @@
         <v>37</v>
       </c>
       <c r="F176">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G176" t="s">
         <v>38</v>
@@ -8507,7 +8507,7 @@
         <v>37</v>
       </c>
       <c r="F177">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="G177" t="s">
         <v>38</v>
@@ -8533,7 +8533,7 @@
         <v>37</v>
       </c>
       <c r="F178">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="G178" t="s">
         <v>38</v>
@@ -8559,7 +8559,7 @@
         <v>37</v>
       </c>
       <c r="F179">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G179" t="s">
         <v>38</v>
@@ -8585,7 +8585,7 @@
         <v>37</v>
       </c>
       <c r="F180">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G180" t="s">
         <v>38</v>
@@ -8611,7 +8611,7 @@
         <v>37</v>
       </c>
       <c r="F181">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="G181" t="s">
         <v>38</v>
@@ -8637,7 +8637,7 @@
         <v>37</v>
       </c>
       <c r="F182">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="G182" t="s">
         <v>38</v>
@@ -8663,7 +8663,7 @@
         <v>37</v>
       </c>
       <c r="F183">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G183" t="s">
         <v>38</v>
@@ -8689,7 +8689,7 @@
         <v>37</v>
       </c>
       <c r="F184">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="G184" t="s">
         <v>38</v>
@@ -8715,7 +8715,7 @@
         <v>37</v>
       </c>
       <c r="F185">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G185" t="s">
         <v>38</v>
@@ -8767,7 +8767,7 @@
         <v>37</v>
       </c>
       <c r="F187">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="G187" t="s">
         <v>38</v>
@@ -8793,7 +8793,7 @@
         <v>37</v>
       </c>
       <c r="F188">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="G188" t="s">
         <v>38</v>
@@ -8819,7 +8819,7 @@
         <v>37</v>
       </c>
       <c r="F189">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="G189" t="s">
         <v>38</v>
@@ -8871,7 +8871,7 @@
         <v>37</v>
       </c>
       <c r="F191">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G191" t="s">
         <v>38</v>
@@ -8897,7 +8897,7 @@
         <v>37</v>
       </c>
       <c r="F192">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="G192" t="s">
         <v>38</v>
@@ -8923,7 +8923,7 @@
         <v>37</v>
       </c>
       <c r="F193">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="G193" t="s">
         <v>38</v>
@@ -8949,7 +8949,7 @@
         <v>37</v>
       </c>
       <c r="F194">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G194" t="s">
         <v>38</v>
@@ -8975,7 +8975,7 @@
         <v>37</v>
       </c>
       <c r="F195">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="G195" t="s">
         <v>38</v>
@@ -9001,7 +9001,7 @@
         <v>37</v>
       </c>
       <c r="F196">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="G196" t="s">
         <v>38</v>
@@ -9027,7 +9027,7 @@
         <v>37</v>
       </c>
       <c r="F197">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G197" t="s">
         <v>38</v>
@@ -9053,7 +9053,7 @@
         <v>37</v>
       </c>
       <c r="F198">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="G198" t="s">
         <v>38</v>
@@ -9079,7 +9079,7 @@
         <v>37</v>
       </c>
       <c r="F199">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="G199" t="s">
         <v>38</v>
@@ -9105,7 +9105,7 @@
         <v>37</v>
       </c>
       <c r="F200">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="G200" t="s">
         <v>38</v>
@@ -9131,7 +9131,7 @@
         <v>37</v>
       </c>
       <c r="F201">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G201" t="s">
         <v>38</v>
@@ -9157,7 +9157,7 @@
         <v>37</v>
       </c>
       <c r="F202">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="G202" t="s">
         <v>38</v>
@@ -9183,7 +9183,7 @@
         <v>37</v>
       </c>
       <c r="F203">
-        <v>19</v>
+        <v>40</v>
       </c>
       <c r="G203" t="s">
         <v>38</v>
@@ -9209,7 +9209,7 @@
         <v>37</v>
       </c>
       <c r="F204">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G204" t="s">
         <v>38</v>
@@ -9235,7 +9235,7 @@
         <v>37</v>
       </c>
       <c r="F205">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G205" t="s">
         <v>38</v>
@@ -9261,7 +9261,7 @@
         <v>37</v>
       </c>
       <c r="F206">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="G206" t="s">
         <v>38</v>
@@ -9287,7 +9287,7 @@
         <v>37</v>
       </c>
       <c r="F207">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="G207" t="s">
         <v>38</v>
@@ -9313,7 +9313,7 @@
         <v>37</v>
       </c>
       <c r="F208">
-        <v>52</v>
+        <v>22</v>
       </c>
       <c r="G208" t="s">
         <v>38</v>
@@ -9339,7 +9339,7 @@
         <v>37</v>
       </c>
       <c r="F209">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="G209" t="s">
         <v>38</v>
@@ -9365,7 +9365,7 @@
         <v>37</v>
       </c>
       <c r="F210">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="G210" t="s">
         <v>38</v>
@@ -9391,7 +9391,7 @@
         <v>37</v>
       </c>
       <c r="F211">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G211" t="s">
         <v>38</v>
@@ -9417,7 +9417,7 @@
         <v>37</v>
       </c>
       <c r="F212">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="G212" t="s">
         <v>38</v>
@@ -9443,7 +9443,7 @@
         <v>37</v>
       </c>
       <c r="F213">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="G213" t="s">
         <v>38</v>
@@ -9469,7 +9469,7 @@
         <v>37</v>
       </c>
       <c r="F214">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="G214" t="s">
         <v>38</v>
@@ -9495,7 +9495,7 @@
         <v>37</v>
       </c>
       <c r="F215">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G215" t="s">
         <v>38</v>
@@ -9521,7 +9521,7 @@
         <v>37</v>
       </c>
       <c r="F216">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="G216" t="s">
         <v>38</v>
@@ -9547,7 +9547,7 @@
         <v>37</v>
       </c>
       <c r="F217">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="G217" t="s">
         <v>38</v>
@@ -9573,7 +9573,7 @@
         <v>37</v>
       </c>
       <c r="F218">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G218" t="s">
         <v>38</v>
@@ -9599,7 +9599,7 @@
         <v>37</v>
       </c>
       <c r="F219">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="G219" t="s">
         <v>38</v>
@@ -9625,7 +9625,7 @@
         <v>37</v>
       </c>
       <c r="F220">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="G220" t="s">
         <v>38</v>
@@ -9651,7 +9651,7 @@
         <v>37</v>
       </c>
       <c r="F221">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G221" t="s">
         <v>38</v>
@@ -9677,7 +9677,7 @@
         <v>37</v>
       </c>
       <c r="F222">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="G222" t="s">
         <v>38</v>
@@ -9703,7 +9703,7 @@
         <v>37</v>
       </c>
       <c r="F223">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="G223" t="s">
         <v>38</v>
@@ -9729,7 +9729,7 @@
         <v>37</v>
       </c>
       <c r="F224">
-        <v>49</v>
+        <v>37</v>
       </c>
       <c r="G224" t="s">
         <v>38</v>
@@ -9755,7 +9755,7 @@
         <v>37</v>
       </c>
       <c r="F225">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G225" t="s">
         <v>38</v>
@@ -9781,7 +9781,7 @@
         <v>37</v>
       </c>
       <c r="F226">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G226" t="s">
         <v>38</v>
@@ -9807,7 +9807,7 @@
         <v>37</v>
       </c>
       <c r="F227">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="G227" t="s">
         <v>38</v>
@@ -9833,7 +9833,7 @@
         <v>37</v>
       </c>
       <c r="F228">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G228" t="s">
         <v>38</v>
@@ -9859,7 +9859,7 @@
         <v>37</v>
       </c>
       <c r="F229">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="G229" t="s">
         <v>38</v>
@@ -9885,7 +9885,7 @@
         <v>37</v>
       </c>
       <c r="F230">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G230" t="s">
         <v>38</v>
@@ -9911,7 +9911,7 @@
         <v>37</v>
       </c>
       <c r="F231">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="G231" t="s">
         <v>38</v>
@@ -9937,7 +9937,7 @@
         <v>37</v>
       </c>
       <c r="F232">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="G232" t="s">
         <v>38</v>
@@ -9963,7 +9963,7 @@
         <v>37</v>
       </c>
       <c r="F233">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="G233" t="s">
         <v>38</v>
@@ -9989,7 +9989,7 @@
         <v>37</v>
       </c>
       <c r="F234">
-        <v>53</v>
+        <v>32</v>
       </c>
       <c r="G234" t="s">
         <v>38</v>
@@ -10015,7 +10015,7 @@
         <v>37</v>
       </c>
       <c r="F235">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="G235" t="s">
         <v>38</v>
@@ -10041,7 +10041,7 @@
         <v>37</v>
       </c>
       <c r="F236">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="G236" t="s">
         <v>38</v>
@@ -10067,7 +10067,7 @@
         <v>37</v>
       </c>
       <c r="F237">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G237" t="s">
         <v>38</v>
@@ -10093,7 +10093,7 @@
         <v>37</v>
       </c>
       <c r="F238">
-        <v>48</v>
+        <v>25</v>
       </c>
       <c r="G238" t="s">
         <v>38</v>
@@ -10119,7 +10119,7 @@
         <v>37</v>
       </c>
       <c r="F239">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="G239" t="s">
         <v>38</v>
@@ -10145,7 +10145,7 @@
         <v>37</v>
       </c>
       <c r="F240">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="G240" t="s">
         <v>38</v>
@@ -10171,7 +10171,7 @@
         <v>37</v>
       </c>
       <c r="F241">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="G241" t="s">
         <v>38</v>
@@ -10197,7 +10197,7 @@
         <v>37</v>
       </c>
       <c r="F242">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G242" t="s">
         <v>38</v>
@@ -10223,7 +10223,7 @@
         <v>37</v>
       </c>
       <c r="F243">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="G243" t="s">
         <v>38</v>
@@ -10249,7 +10249,7 @@
         <v>37</v>
       </c>
       <c r="F244">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="G244" t="s">
         <v>38</v>
@@ -10275,7 +10275,7 @@
         <v>37</v>
       </c>
       <c r="F245">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="G245" t="s">
         <v>38</v>
@@ -10301,7 +10301,7 @@
         <v>37</v>
       </c>
       <c r="F246">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="G246" t="s">
         <v>38</v>
@@ -10327,7 +10327,7 @@
         <v>37</v>
       </c>
       <c r="F247">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G247" t="s">
         <v>38</v>
@@ -10353,7 +10353,7 @@
         <v>37</v>
       </c>
       <c r="F248">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="G248" t="s">
         <v>38</v>
@@ -10379,7 +10379,7 @@
         <v>37</v>
       </c>
       <c r="F249">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="G249" t="s">
         <v>38</v>
@@ -10431,7 +10431,7 @@
         <v>37</v>
       </c>
       <c r="F251">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G251" t="s">
         <v>38</v>
@@ -10457,7 +10457,7 @@
         <v>37</v>
       </c>
       <c r="F252">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G252" t="s">
         <v>38</v>
@@ -10483,7 +10483,7 @@
         <v>37</v>
       </c>
       <c r="F253">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="G253" t="s">
         <v>38</v>
@@ -10509,7 +10509,7 @@
         <v>37</v>
       </c>
       <c r="F254">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G254" t="s">
         <v>38</v>
@@ -10561,7 +10561,7 @@
         <v>37</v>
       </c>
       <c r="F256">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G256" t="s">
         <v>38</v>
@@ -10587,7 +10587,7 @@
         <v>37</v>
       </c>
       <c r="F257">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="G257" t="s">
         <v>38</v>
@@ -10613,7 +10613,7 @@
         <v>37</v>
       </c>
       <c r="F258">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="G258" t="s">
         <v>38</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="F259">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="G259" t="s">
         <v>38</v>
@@ -10665,7 +10665,7 @@
         <v>37</v>
       </c>
       <c r="F260">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G260" t="s">
         <v>38</v>
@@ -10691,7 +10691,7 @@
         <v>37</v>
       </c>
       <c r="F261">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="G261" t="s">
         <v>38</v>
@@ -10717,7 +10717,7 @@
         <v>37</v>
       </c>
       <c r="F262">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G262" t="s">
         <v>38</v>
@@ -10743,7 +10743,7 @@
         <v>37</v>
       </c>
       <c r="F263">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="G263" t="s">
         <v>38</v>
@@ -10769,7 +10769,7 @@
         <v>37</v>
       </c>
       <c r="F264">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G264" t="s">
         <v>38</v>
@@ -10795,7 +10795,7 @@
         <v>37</v>
       </c>
       <c r="F265">
-        <v>50</v>
+        <v>24</v>
       </c>
       <c r="G265" t="s">
         <v>38</v>
@@ -10821,7 +10821,7 @@
         <v>37</v>
       </c>
       <c r="F266">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="G266" t="s">
         <v>38</v>
@@ -10847,7 +10847,7 @@
         <v>37</v>
       </c>
       <c r="F267">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="G267" t="s">
         <v>38</v>
@@ -10873,7 +10873,7 @@
         <v>37</v>
       </c>
       <c r="F268">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="G268" t="s">
         <v>38</v>
@@ -10899,7 +10899,7 @@
         <v>37</v>
       </c>
       <c r="F269">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="G269" t="s">
         <v>38</v>
@@ -10925,7 +10925,7 @@
         <v>37</v>
       </c>
       <c r="F270">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="G270" t="s">
         <v>38</v>
@@ -10951,7 +10951,7 @@
         <v>37</v>
       </c>
       <c r="F271">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G271" t="s">
         <v>38</v>
@@ -10977,7 +10977,7 @@
         <v>37</v>
       </c>
       <c r="F272">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="G272" t="s">
         <v>38</v>
@@ -11003,7 +11003,7 @@
         <v>37</v>
       </c>
       <c r="F273">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="G273" t="s">
         <v>38</v>
@@ -11029,7 +11029,7 @@
         <v>37</v>
       </c>
       <c r="F274">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="G274" t="s">
         <v>38</v>
@@ -11055,7 +11055,7 @@
         <v>37</v>
       </c>
       <c r="F275">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G275" t="s">
         <v>38</v>
@@ -11081,7 +11081,7 @@
         <v>37</v>
       </c>
       <c r="F276">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G276" t="s">
         <v>38</v>
@@ -11107,7 +11107,7 @@
         <v>37</v>
       </c>
       <c r="F277">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G277" t="s">
         <v>38</v>
@@ -11133,7 +11133,7 @@
         <v>37</v>
       </c>
       <c r="F278">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G278" t="s">
         <v>38</v>
@@ -11159,7 +11159,7 @@
         <v>37</v>
       </c>
       <c r="F279">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="G279" t="s">
         <v>38</v>
@@ -11185,7 +11185,7 @@
         <v>37</v>
       </c>
       <c r="F280">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="G280" t="s">
         <v>38</v>
@@ -11211,7 +11211,7 @@
         <v>37</v>
       </c>
       <c r="F281">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="G281" t="s">
         <v>38</v>
@@ -11263,7 +11263,7 @@
         <v>37</v>
       </c>
       <c r="F283">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G283" t="s">
         <v>38</v>
@@ -11289,7 +11289,7 @@
         <v>37</v>
       </c>
       <c r="F284">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G284" t="s">
         <v>38</v>
@@ -11315,7 +11315,7 @@
         <v>37</v>
       </c>
       <c r="F285">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G285" t="s">
         <v>38</v>
@@ -11341,7 +11341,7 @@
         <v>37</v>
       </c>
       <c r="F286">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="G286" t="s">
         <v>38</v>
@@ -11367,7 +11367,7 @@
         <v>37</v>
       </c>
       <c r="F287">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="G287" t="s">
         <v>38</v>
@@ -11393,7 +11393,7 @@
         <v>37</v>
       </c>
       <c r="F288">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="G288" t="s">
         <v>38</v>
@@ -11419,7 +11419,7 @@
         <v>37</v>
       </c>
       <c r="F289">
-        <v>51</v>
+        <v>19</v>
       </c>
       <c r="G289" t="s">
         <v>38</v>
@@ -11445,7 +11445,7 @@
         <v>37</v>
       </c>
       <c r="F290">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G290" t="s">
         <v>38</v>
@@ -11471,7 +11471,7 @@
         <v>37</v>
       </c>
       <c r="F291">
-        <v>31</v>
+        <v>15</v>
       </c>
       <c r="G291" t="s">
         <v>38</v>
@@ -11497,7 +11497,7 @@
         <v>37</v>
       </c>
       <c r="F292">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="G292" t="s">
         <v>38</v>
@@ -11523,7 +11523,7 @@
         <v>37</v>
       </c>
       <c r="F293">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G293" t="s">
         <v>38</v>
@@ -11549,7 +11549,7 @@
         <v>37</v>
       </c>
       <c r="F294">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="G294" t="s">
         <v>38</v>
@@ -11575,7 +11575,7 @@
         <v>37</v>
       </c>
       <c r="F295">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="G295" t="s">
         <v>38</v>
@@ -11601,7 +11601,7 @@
         <v>37</v>
       </c>
       <c r="F296">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G296" t="s">
         <v>38</v>
@@ -11653,7 +11653,7 @@
         <v>37</v>
       </c>
       <c r="F298">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="G298" t="s">
         <v>38</v>
@@ -11679,7 +11679,7 @@
         <v>37</v>
       </c>
       <c r="F299">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G299" t="s">
         <v>38</v>
@@ -11705,7 +11705,7 @@
         <v>37</v>
       </c>
       <c r="F300">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="G300" t="s">
         <v>38</v>
@@ -11757,7 +11757,7 @@
         <v>37</v>
       </c>
       <c r="F302">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="G302" t="s">
         <v>38</v>
@@ -11783,7 +11783,7 @@
         <v>37</v>
       </c>
       <c r="F303">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G303" t="s">
         <v>38</v>
@@ -11809,7 +11809,7 @@
         <v>37</v>
       </c>
       <c r="F304">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="G304" t="s">
         <v>38</v>
@@ -11835,7 +11835,7 @@
         <v>37</v>
       </c>
       <c r="F305">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G305" t="s">
         <v>38</v>
@@ -11861,7 +11861,7 @@
         <v>37</v>
       </c>
       <c r="F306">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="G306" t="s">
         <v>38</v>
@@ -11887,7 +11887,7 @@
         <v>37</v>
       </c>
       <c r="F307">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G307" t="s">
         <v>38</v>
@@ -11913,7 +11913,7 @@
         <v>37</v>
       </c>
       <c r="F308">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="G308" t="s">
         <v>38</v>
@@ -11939,7 +11939,7 @@
         <v>37</v>
       </c>
       <c r="F309">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="G309" t="s">
         <v>38</v>
@@ -11965,7 +11965,7 @@
         <v>37</v>
       </c>
       <c r="F310">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="G310" t="s">
         <v>38</v>
@@ -11991,7 +11991,7 @@
         <v>37</v>
       </c>
       <c r="F311">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="G311" t="s">
         <v>38</v>
@@ -12017,7 +12017,7 @@
         <v>37</v>
       </c>
       <c r="F312">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G312" t="s">
         <v>38</v>
@@ -12043,7 +12043,7 @@
         <v>37</v>
       </c>
       <c r="F313">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="G313" t="s">
         <v>38</v>
@@ -12069,7 +12069,7 @@
         <v>37</v>
       </c>
       <c r="F314">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="G314" t="s">
         <v>38</v>
@@ -12095,7 +12095,7 @@
         <v>37</v>
       </c>
       <c r="F315">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="G315" t="s">
         <v>38</v>
@@ -12121,7 +12121,7 @@
         <v>37</v>
       </c>
       <c r="F316">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="G316" t="s">
         <v>38</v>
@@ -12147,7 +12147,7 @@
         <v>37</v>
       </c>
       <c r="F317">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="G317" t="s">
         <v>38</v>
@@ -12173,7 +12173,7 @@
         <v>37</v>
       </c>
       <c r="F318">
-        <v>34</v>
+        <v>50</v>
       </c>
       <c r="G318" t="s">
         <v>38</v>
@@ -12199,7 +12199,7 @@
         <v>37</v>
       </c>
       <c r="F319">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G319" t="s">
         <v>38</v>
@@ -12225,7 +12225,7 @@
         <v>37</v>
       </c>
       <c r="F320">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="G320" t="s">
         <v>38</v>
@@ -12251,7 +12251,7 @@
         <v>37</v>
       </c>
       <c r="F321">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="G321" t="s">
         <v>38</v>
@@ -12277,7 +12277,7 @@
         <v>37</v>
       </c>
       <c r="F322">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="G322" t="s">
         <v>38</v>
@@ -12303,7 +12303,7 @@
         <v>37</v>
       </c>
       <c r="F323">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="G323" t="s">
         <v>38</v>
@@ -12329,7 +12329,7 @@
         <v>37</v>
       </c>
       <c r="F324">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G324" t="s">
         <v>38</v>
@@ -12355,7 +12355,7 @@
         <v>37</v>
       </c>
       <c r="F325">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="G325" t="s">
         <v>38</v>
@@ -12381,7 +12381,7 @@
         <v>37</v>
       </c>
       <c r="F326">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G326" t="s">
         <v>38</v>
@@ -12407,7 +12407,7 @@
         <v>37</v>
       </c>
       <c r="F327">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G327" t="s">
         <v>38</v>
@@ -12459,7 +12459,7 @@
         <v>37</v>
       </c>
       <c r="F329">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="G329" t="s">
         <v>38</v>
@@ -12485,7 +12485,7 @@
         <v>37</v>
       </c>
       <c r="F330">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="G330" t="s">
         <v>38</v>
@@ -12511,7 +12511,7 @@
         <v>37</v>
       </c>
       <c r="F331">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="G331" t="s">
         <v>38</v>
@@ -12537,7 +12537,7 @@
         <v>37</v>
       </c>
       <c r="F332">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="G332" t="s">
         <v>38</v>
@@ -12563,7 +12563,7 @@
         <v>37</v>
       </c>
       <c r="F333">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G333" t="s">
         <v>38</v>
@@ -12589,7 +12589,7 @@
         <v>37</v>
       </c>
       <c r="F334">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="G334" t="s">
         <v>38</v>
@@ -12641,7 +12641,7 @@
         <v>37</v>
       </c>
       <c r="F336">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="G336" t="s">
         <v>38</v>
@@ -12667,7 +12667,7 @@
         <v>37</v>
       </c>
       <c r="F337">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G337" t="s">
         <v>38</v>
@@ -12693,7 +12693,7 @@
         <v>37</v>
       </c>
       <c r="F338">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="G338" t="s">
         <v>38</v>
@@ -12719,7 +12719,7 @@
         <v>37</v>
       </c>
       <c r="F339">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="G339" t="s">
         <v>38</v>
@@ -12745,7 +12745,7 @@
         <v>37</v>
       </c>
       <c r="F340">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G340" t="s">
         <v>38</v>
@@ -12771,7 +12771,7 @@
         <v>37</v>
       </c>
       <c r="F341">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G341" t="s">
         <v>38</v>
@@ -12797,7 +12797,7 @@
         <v>37</v>
       </c>
       <c r="F342">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G342" t="s">
         <v>38</v>
@@ -12823,7 +12823,7 @@
         <v>37</v>
       </c>
       <c r="F343">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="G343" t="s">
         <v>38</v>
@@ -12849,7 +12849,7 @@
         <v>37</v>
       </c>
       <c r="F344">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="G344" t="s">
         <v>38</v>
@@ -12875,7 +12875,7 @@
         <v>37</v>
       </c>
       <c r="F345">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="G345" t="s">
         <v>38</v>
@@ -12901,7 +12901,7 @@
         <v>37</v>
       </c>
       <c r="F346">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G346" t="s">
         <v>38</v>
@@ -12927,7 +12927,7 @@
         <v>37</v>
       </c>
       <c r="F347">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="G347" t="s">
         <v>38</v>
@@ -12953,7 +12953,7 @@
         <v>37</v>
       </c>
       <c r="F348">
-        <v>23</v>
+        <v>49</v>
       </c>
       <c r="G348" t="s">
         <v>38</v>
@@ -12979,7 +12979,7 @@
         <v>37</v>
       </c>
       <c r="F349">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G349" t="s">
         <v>38</v>
@@ -13005,7 +13005,7 @@
         <v>37</v>
       </c>
       <c r="F350">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="G350" t="s">
         <v>38</v>
@@ -13031,7 +13031,7 @@
         <v>37</v>
       </c>
       <c r="F351">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G351" t="s">
         <v>38</v>
@@ -13057,7 +13057,7 @@
         <v>37</v>
       </c>
       <c r="F352">
-        <v>54</v>
+        <v>33</v>
       </c>
       <c r="G352" t="s">
         <v>38</v>
@@ -13083,7 +13083,7 @@
         <v>37</v>
       </c>
       <c r="F353">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="G353" t="s">
         <v>38</v>
@@ -13109,7 +13109,7 @@
         <v>37</v>
       </c>
       <c r="F354">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G354" t="s">
         <v>38</v>
@@ -13135,7 +13135,7 @@
         <v>37</v>
       </c>
       <c r="F355">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G355" t="s">
         <v>38</v>
@@ -13161,7 +13161,7 @@
         <v>37</v>
       </c>
       <c r="F356">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="G356" t="s">
         <v>38</v>
@@ -13187,7 +13187,7 @@
         <v>37</v>
       </c>
       <c r="F357">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G357" t="s">
         <v>38</v>
@@ -13213,7 +13213,7 @@
         <v>37</v>
       </c>
       <c r="F358">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G358" t="s">
         <v>38</v>
@@ -13239,7 +13239,7 @@
         <v>37</v>
       </c>
       <c r="F359">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G359" t="s">
         <v>38</v>
@@ -13265,7 +13265,7 @@
         <v>37</v>
       </c>
       <c r="F360">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="G360" t="s">
         <v>38</v>
@@ -13291,7 +13291,7 @@
         <v>37</v>
       </c>
       <c r="F361">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="G361" t="s">
         <v>38</v>
@@ -13317,7 +13317,7 @@
         <v>37</v>
       </c>
       <c r="F362">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="G362" t="s">
         <v>38</v>
@@ -13343,7 +13343,7 @@
         <v>37</v>
       </c>
       <c r="F363">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="G363" t="s">
         <v>38</v>
@@ -13369,7 +13369,7 @@
         <v>37</v>
       </c>
       <c r="F364">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="G364" t="s">
         <v>38</v>
@@ -13395,7 +13395,7 @@
         <v>37</v>
       </c>
       <c r="F365">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="G365" t="s">
         <v>38</v>
@@ -13421,7 +13421,7 @@
         <v>37</v>
       </c>
       <c r="F366">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="G366" t="s">
         <v>38</v>
@@ -13447,7 +13447,7 @@
         <v>37</v>
       </c>
       <c r="F367">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G367" t="s">
         <v>38</v>
@@ -13473,7 +13473,7 @@
         <v>37</v>
       </c>
       <c r="F368">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G368" t="s">
         <v>38</v>
@@ -13499,7 +13499,7 @@
         <v>37</v>
       </c>
       <c r="F369">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="G369" t="s">
         <v>38</v>
@@ -13525,7 +13525,7 @@
         <v>37</v>
       </c>
       <c r="F370">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G370" t="s">
         <v>38</v>
@@ -13551,7 +13551,7 @@
         <v>37</v>
       </c>
       <c r="F371">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G371" t="s">
         <v>38</v>
@@ -13577,7 +13577,7 @@
         <v>37</v>
       </c>
       <c r="F372">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="G372" t="s">
         <v>38</v>
@@ -13603,7 +13603,7 @@
         <v>37</v>
       </c>
       <c r="F373">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G373" t="s">
         <v>38</v>
@@ -13629,7 +13629,7 @@
         <v>37</v>
       </c>
       <c r="F374">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G374" t="s">
         <v>38</v>
@@ -13655,7 +13655,7 @@
         <v>37</v>
       </c>
       <c r="F375">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="G375" t="s">
         <v>38</v>
@@ -13681,7 +13681,7 @@
         <v>37</v>
       </c>
       <c r="F376">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="G376" t="s">
         <v>38</v>
@@ -13707,7 +13707,7 @@
         <v>37</v>
       </c>
       <c r="F377">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="G377" t="s">
         <v>38</v>
@@ -13733,7 +13733,7 @@
         <v>37</v>
       </c>
       <c r="F378">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="G378" t="s">
         <v>38</v>
@@ -13759,7 +13759,7 @@
         <v>37</v>
       </c>
       <c r="F379">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G379" t="s">
         <v>38</v>
@@ -13785,7 +13785,7 @@
         <v>37</v>
       </c>
       <c r="F380">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="G380" t="s">
         <v>38</v>
@@ -13811,7 +13811,7 @@
         <v>37</v>
       </c>
       <c r="F381">
-        <v>53</v>
+        <v>19</v>
       </c>
       <c r="G381" t="s">
         <v>38</v>
@@ -13837,7 +13837,7 @@
         <v>37</v>
       </c>
       <c r="F382">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G382" t="s">
         <v>38</v>
@@ -13863,7 +13863,7 @@
         <v>37</v>
       </c>
       <c r="F383">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G383" t="s">
         <v>38</v>
@@ -13889,7 +13889,7 @@
         <v>37</v>
       </c>
       <c r="F384">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="G384" t="s">
         <v>38</v>
@@ -13915,7 +13915,7 @@
         <v>37</v>
       </c>
       <c r="F385">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G385" t="s">
         <v>38</v>
@@ -13941,7 +13941,7 @@
         <v>37</v>
       </c>
       <c r="F386">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G386" t="s">
         <v>38</v>
@@ -13967,7 +13967,7 @@
         <v>37</v>
       </c>
       <c r="F387">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="G387" t="s">
         <v>38</v>
@@ -13993,7 +13993,7 @@
         <v>37</v>
       </c>
       <c r="F388">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G388" t="s">
         <v>38</v>
@@ -14019,7 +14019,7 @@
         <v>37</v>
       </c>
       <c r="F389">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G389" t="s">
         <v>38</v>
@@ -14045,7 +14045,7 @@
         <v>37</v>
       </c>
       <c r="F390">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G390" t="s">
         <v>38</v>
@@ -14071,7 +14071,7 @@
         <v>37</v>
       </c>
       <c r="F391">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="G391" t="s">
         <v>38</v>
@@ -14097,7 +14097,7 @@
         <v>37</v>
       </c>
       <c r="F392">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G392" t="s">
         <v>38</v>
@@ -14123,7 +14123,7 @@
         <v>37</v>
       </c>
       <c r="F393">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="G393" t="s">
         <v>38</v>
@@ -14149,7 +14149,7 @@
         <v>37</v>
       </c>
       <c r="F394">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="G394" t="s">
         <v>38</v>
@@ -14175,7 +14175,7 @@
         <v>37</v>
       </c>
       <c r="F395">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G395" t="s">
         <v>38</v>
@@ -14201,7 +14201,7 @@
         <v>37</v>
       </c>
       <c r="F396">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G396" t="s">
         <v>38</v>
@@ -14227,7 +14227,7 @@
         <v>37</v>
       </c>
       <c r="F397">
-        <v>52</v>
+        <v>16</v>
       </c>
       <c r="G397" t="s">
         <v>38</v>
@@ -14253,7 +14253,7 @@
         <v>37</v>
       </c>
       <c r="F398">
-        <v>26</v>
+        <v>49</v>
       </c>
       <c r="G398" t="s">
         <v>38</v>
@@ -14279,7 +14279,7 @@
         <v>37</v>
       </c>
       <c r="F399">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="G399" t="s">
         <v>38</v>
@@ -14305,7 +14305,7 @@
         <v>37</v>
       </c>
       <c r="F400">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="G400" t="s">
         <v>38</v>
@@ -14331,7 +14331,7 @@
         <v>37</v>
       </c>
       <c r="F401">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="G401" t="s">
         <v>38</v>
@@ -14357,7 +14357,7 @@
         <v>37</v>
       </c>
       <c r="F402">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="G402" t="s">
         <v>38</v>
@@ -14383,7 +14383,7 @@
         <v>37</v>
       </c>
       <c r="F403">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="G403" t="s">
         <v>38</v>
@@ -14409,7 +14409,7 @@
         <v>37</v>
       </c>
       <c r="F404">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="G404" t="s">
         <v>38</v>
@@ -14435,7 +14435,7 @@
         <v>37</v>
       </c>
       <c r="F405">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G405" t="s">
         <v>38</v>
@@ -14461,7 +14461,7 @@
         <v>37</v>
       </c>
       <c r="F406">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="G406" t="s">
         <v>38</v>
@@ -14487,7 +14487,7 @@
         <v>37</v>
       </c>
       <c r="F407">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="G407" t="s">
         <v>38</v>
@@ -14513,7 +14513,7 @@
         <v>37</v>
       </c>
       <c r="F408">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G408" t="s">
         <v>38</v>
@@ -14539,7 +14539,7 @@
         <v>37</v>
       </c>
       <c r="F409">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="G409" t="s">
         <v>38</v>
@@ -14565,7 +14565,7 @@
         <v>37</v>
       </c>
       <c r="F410">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G410" t="s">
         <v>38</v>
@@ -14591,7 +14591,7 @@
         <v>37</v>
       </c>
       <c r="F411">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="G411" t="s">
         <v>38</v>
@@ -14617,7 +14617,7 @@
         <v>37</v>
       </c>
       <c r="F412">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="G412" t="s">
         <v>38</v>
@@ -14643,7 +14643,7 @@
         <v>37</v>
       </c>
       <c r="F413">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="G413" t="s">
         <v>38</v>
@@ -14669,7 +14669,7 @@
         <v>37</v>
       </c>
       <c r="F414">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G414" t="s">
         <v>38</v>
@@ -14695,7 +14695,7 @@
         <v>37</v>
       </c>
       <c r="F415">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G415" t="s">
         <v>38</v>
@@ -14721,7 +14721,7 @@
         <v>37</v>
       </c>
       <c r="F416">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G416" t="s">
         <v>38</v>
@@ -14747,7 +14747,7 @@
         <v>37</v>
       </c>
       <c r="F417">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="G417" t="s">
         <v>38</v>
@@ -14773,7 +14773,7 @@
         <v>37</v>
       </c>
       <c r="F418">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="G418" t="s">
         <v>38</v>
@@ -14799,7 +14799,7 @@
         <v>37</v>
       </c>
       <c r="F419">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G419" t="s">
         <v>38</v>
@@ -14825,7 +14825,7 @@
         <v>37</v>
       </c>
       <c r="F420">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G420" t="s">
         <v>38</v>
@@ -14851,7 +14851,7 @@
         <v>37</v>
       </c>
       <c r="F421">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G421" t="s">
         <v>38</v>
@@ -14877,7 +14877,7 @@
         <v>37</v>
       </c>
       <c r="F422">
-        <v>27</v>
+        <v>50</v>
       </c>
       <c r="G422" t="s">
         <v>38</v>
@@ -14903,7 +14903,7 @@
         <v>37</v>
       </c>
       <c r="F423">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="G423" t="s">
         <v>38</v>
@@ -14929,7 +14929,7 @@
         <v>37</v>
       </c>
       <c r="F424">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="G424" t="s">
         <v>38</v>
@@ -14955,7 +14955,7 @@
         <v>37</v>
       </c>
       <c r="F425">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G425" t="s">
         <v>38</v>
@@ -14981,7 +14981,7 @@
         <v>37</v>
       </c>
       <c r="F426">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="G426" t="s">
         <v>38</v>
@@ -15007,7 +15007,7 @@
         <v>37</v>
       </c>
       <c r="F427">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G427" t="s">
         <v>38</v>
@@ -15033,7 +15033,7 @@
         <v>37</v>
       </c>
       <c r="F428">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="G428" t="s">
         <v>38</v>
@@ -15059,7 +15059,7 @@
         <v>37</v>
       </c>
       <c r="F429">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="G429" t="s">
         <v>38</v>
@@ -15085,7 +15085,7 @@
         <v>37</v>
       </c>
       <c r="F430">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G430" t="s">
         <v>38</v>
@@ -15111,7 +15111,7 @@
         <v>37</v>
       </c>
       <c r="F431">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G431" t="s">
         <v>38</v>
@@ -15137,7 +15137,7 @@
         <v>37</v>
       </c>
       <c r="F432">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="G432" t="s">
         <v>38</v>
@@ -15163,7 +15163,7 @@
         <v>37</v>
       </c>
       <c r="F433">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G433" t="s">
         <v>38</v>
@@ -15189,7 +15189,7 @@
         <v>37</v>
       </c>
       <c r="F434">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="G434" t="s">
         <v>38</v>
@@ -15241,7 +15241,7 @@
         <v>37</v>
       </c>
       <c r="F436">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="G436" t="s">
         <v>38</v>
@@ -15267,7 +15267,7 @@
         <v>37</v>
       </c>
       <c r="F437">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="G437" t="s">
         <v>38</v>
@@ -15293,7 +15293,7 @@
         <v>37</v>
       </c>
       <c r="F438">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="G438" t="s">
         <v>38</v>
@@ -15319,7 +15319,7 @@
         <v>37</v>
       </c>
       <c r="F439">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G439" t="s">
         <v>38</v>
@@ -15345,7 +15345,7 @@
         <v>37</v>
       </c>
       <c r="F440">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G440" t="s">
         <v>38</v>
@@ -15371,7 +15371,7 @@
         <v>37</v>
       </c>
       <c r="F441">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="G441" t="s">
         <v>38</v>
@@ -15397,7 +15397,7 @@
         <v>37</v>
       </c>
       <c r="F442">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="G442" t="s">
         <v>38</v>
@@ -15423,7 +15423,7 @@
         <v>37</v>
       </c>
       <c r="F443">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G443" t="s">
         <v>38</v>
@@ -15449,7 +15449,7 @@
         <v>37</v>
       </c>
       <c r="F444">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="G444" t="s">
         <v>38</v>
@@ -15475,7 +15475,7 @@
         <v>37</v>
       </c>
       <c r="F445">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G445" t="s">
         <v>38</v>
@@ -15501,7 +15501,7 @@
         <v>37</v>
       </c>
       <c r="F446">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="G446" t="s">
         <v>38</v>
@@ -15527,7 +15527,7 @@
         <v>37</v>
       </c>
       <c r="F447">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="G447" t="s">
         <v>38</v>
@@ -15553,7 +15553,7 @@
         <v>37</v>
       </c>
       <c r="F448">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="G448" t="s">
         <v>38</v>
@@ -15579,7 +15579,7 @@
         <v>37</v>
       </c>
       <c r="F449">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="G449" t="s">
         <v>38</v>
@@ -15605,7 +15605,7 @@
         <v>37</v>
       </c>
       <c r="F450">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G450" t="s">
         <v>38</v>
@@ -15631,7 +15631,7 @@
         <v>37</v>
       </c>
       <c r="F451">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="G451" t="s">
         <v>38</v>
@@ -15657,7 +15657,7 @@
         <v>37</v>
       </c>
       <c r="F452">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="G452" t="s">
         <v>38</v>
@@ -15683,7 +15683,7 @@
         <v>37</v>
       </c>
       <c r="F453">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G453" t="s">
         <v>38</v>
@@ -15709,7 +15709,7 @@
         <v>37</v>
       </c>
       <c r="F454">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="G454" t="s">
         <v>38</v>
@@ -15735,7 +15735,7 @@
         <v>37</v>
       </c>
       <c r="F455">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G455" t="s">
         <v>38</v>
@@ -15761,7 +15761,7 @@
         <v>37</v>
       </c>
       <c r="F456">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G456" t="s">
         <v>38</v>
@@ -15787,7 +15787,7 @@
         <v>37</v>
       </c>
       <c r="F457">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="G457" t="s">
         <v>38</v>
@@ -15813,7 +15813,7 @@
         <v>37</v>
       </c>
       <c r="F458">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="G458" t="s">
         <v>38</v>
@@ -15839,7 +15839,7 @@
         <v>37</v>
       </c>
       <c r="F459">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="G459" t="s">
         <v>38</v>
@@ -15865,7 +15865,7 @@
         <v>37</v>
       </c>
       <c r="F460">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="G460" t="s">
         <v>38</v>
@@ -15891,7 +15891,7 @@
         <v>37</v>
       </c>
       <c r="F461">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="G461" t="s">
         <v>38</v>
@@ -15917,7 +15917,7 @@
         <v>37</v>
       </c>
       <c r="F462">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G462" t="s">
         <v>38</v>
@@ -15943,7 +15943,7 @@
         <v>37</v>
       </c>
       <c r="F463">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G463" t="s">
         <v>38</v>
@@ -15969,7 +15969,7 @@
         <v>37</v>
       </c>
       <c r="F464">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="G464" t="s">
         <v>38</v>
@@ -15995,7 +15995,7 @@
         <v>37</v>
       </c>
       <c r="F465">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G465" t="s">
         <v>38</v>
@@ -16021,7 +16021,7 @@
         <v>37</v>
       </c>
       <c r="F466">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G466" t="s">
         <v>38</v>
@@ -16047,7 +16047,7 @@
         <v>37</v>
       </c>
       <c r="F467">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="G467" t="s">
         <v>38</v>
@@ -16073,7 +16073,7 @@
         <v>37</v>
       </c>
       <c r="F468">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="G468" t="s">
         <v>38</v>
@@ -16099,7 +16099,7 @@
         <v>37</v>
       </c>
       <c r="F469">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="G469" t="s">
         <v>38</v>
@@ -16125,7 +16125,7 @@
         <v>37</v>
       </c>
       <c r="F470">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="G470" t="s">
         <v>38</v>
@@ -16151,7 +16151,7 @@
         <v>37</v>
       </c>
       <c r="F471">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G471" t="s">
         <v>38</v>
@@ -16177,7 +16177,7 @@
         <v>37</v>
       </c>
       <c r="F472">
-        <v>22</v>
+        <v>49</v>
       </c>
       <c r="G472" t="s">
         <v>38</v>
@@ -16203,7 +16203,7 @@
         <v>37</v>
       </c>
       <c r="F473">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G473" t="s">
         <v>38</v>
@@ -16229,7 +16229,7 @@
         <v>37</v>
       </c>
       <c r="F474">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="G474" t="s">
         <v>38</v>
@@ -16255,7 +16255,7 @@
         <v>37</v>
       </c>
       <c r="F475">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="G475" t="s">
         <v>38</v>
@@ -16281,7 +16281,7 @@
         <v>37</v>
       </c>
       <c r="F476">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G476" t="s">
         <v>38</v>
@@ -16307,7 +16307,7 @@
         <v>37</v>
       </c>
       <c r="F477">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="G477" t="s">
         <v>38</v>
@@ -16333,7 +16333,7 @@
         <v>37</v>
       </c>
       <c r="F478">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="G478" t="s">
         <v>38</v>
@@ -16359,7 +16359,7 @@
         <v>37</v>
       </c>
       <c r="F479">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="G479" t="s">
         <v>38</v>
@@ -16385,7 +16385,7 @@
         <v>37</v>
       </c>
       <c r="F480">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G480" t="s">
         <v>38</v>
@@ -16411,7 +16411,7 @@
         <v>37</v>
       </c>
       <c r="F481">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="G481" t="s">
         <v>38</v>
@@ -16437,7 +16437,7 @@
         <v>37</v>
       </c>
       <c r="F482">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="G482" t="s">
         <v>38</v>
@@ -16463,7 +16463,7 @@
         <v>37</v>
       </c>
       <c r="F483">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="G483" t="s">
         <v>38</v>
@@ -16489,7 +16489,7 @@
         <v>37</v>
       </c>
       <c r="F484">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G484" t="s">
         <v>38</v>
@@ -16515,7 +16515,7 @@
         <v>37</v>
       </c>
       <c r="F485">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="G485" t="s">
         <v>38</v>
@@ -16541,7 +16541,7 @@
         <v>37</v>
       </c>
       <c r="F486">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="G486" t="s">
         <v>38</v>
@@ -16567,7 +16567,7 @@
         <v>37</v>
       </c>
       <c r="F487">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="G487" t="s">
         <v>38</v>
@@ -16593,7 +16593,7 @@
         <v>37</v>
       </c>
       <c r="F488">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G488" t="s">
         <v>38</v>
@@ -16619,7 +16619,7 @@
         <v>37</v>
       </c>
       <c r="F489">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="G489" t="s">
         <v>38</v>
@@ -16645,7 +16645,7 @@
         <v>37</v>
       </c>
       <c r="F490">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="G490" t="s">
         <v>38</v>
@@ -16671,7 +16671,7 @@
         <v>37</v>
       </c>
       <c r="F491">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G491" t="s">
         <v>38</v>
@@ -16697,7 +16697,7 @@
         <v>37</v>
       </c>
       <c r="F492">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="G492" t="s">
         <v>38</v>
@@ -16723,7 +16723,7 @@
         <v>37</v>
       </c>
       <c r="F493">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G493" t="s">
         <v>38</v>
@@ -16749,7 +16749,7 @@
         <v>37</v>
       </c>
       <c r="F494">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G494" t="s">
         <v>38</v>
@@ -16775,7 +16775,7 @@
         <v>37</v>
       </c>
       <c r="F495">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G495" t="s">
         <v>38</v>
@@ -16801,7 +16801,7 @@
         <v>37</v>
       </c>
       <c r="F496">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="G496" t="s">
         <v>38</v>
@@ -16827,7 +16827,7 @@
         <v>37</v>
       </c>
       <c r="F497">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="G497" t="s">
         <v>38</v>
@@ -16853,7 +16853,7 @@
         <v>37</v>
       </c>
       <c r="F498">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G498" t="s">
         <v>38</v>
@@ -16879,7 +16879,7 @@
         <v>37</v>
       </c>
       <c r="F499">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G499" t="s">
         <v>38</v>
@@ -16905,7 +16905,7 @@
         <v>37</v>
       </c>
       <c r="F500">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="G500" t="s">
         <v>38</v>
@@ -16931,7 +16931,7 @@
         <v>37</v>
       </c>
       <c r="F501">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G501" t="s">
         <v>38</v>

</xml_diff>

<commit_message>
Complete NGO dashboard overhaul with stats cards, status filters, active requirements, and tracking on mobile
</commit_message>
<xml_diff>
--- a/e2e-tests/reports/test-report.xlsx
+++ b/e2e-tests/reports/test-report.xlsx
@@ -42,19 +42,19 @@
     <t>Total Execution Time</t>
   </si>
   <si>
-    <t>17.19s</t>
+    <t>17.54s</t>
   </si>
   <si>
     <t>Average Test Duration</t>
   </si>
   <si>
-    <t>34.37ms</t>
+    <t>35.08ms</t>
   </si>
   <si>
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>7/23/2026, 3:23:00 PM</t>
+    <t>7/23/2026, 3:53:34 PM</t>
   </si>
   <si>
     <t>Category</t>
@@ -3684,7 +3684,7 @@
         <v>100</v>
       </c>
       <c r="G2">
-        <v>34.46</v>
+        <v>35.66</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -3707,7 +3707,7 @@
         <v>100</v>
       </c>
       <c r="G3">
-        <v>34.24</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -3730,7 +3730,7 @@
         <v>100</v>
       </c>
       <c r="G4">
-        <v>35.46</v>
+        <v>35.74</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -3753,7 +3753,7 @@
         <v>100</v>
       </c>
       <c r="G5">
-        <v>33.54</v>
+        <v>34.46</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -3776,7 +3776,7 @@
         <v>100</v>
       </c>
       <c r="G6">
-        <v>36.26</v>
+        <v>33.18</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -3799,7 +3799,7 @@
         <v>100</v>
       </c>
       <c r="G7">
-        <v>33.88</v>
+        <v>33.82</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -3822,7 +3822,7 @@
         <v>100</v>
       </c>
       <c r="G8">
-        <v>34.64</v>
+        <v>34.48</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -3845,7 +3845,7 @@
         <v>100</v>
       </c>
       <c r="G9">
-        <v>31.58</v>
+        <v>34.52</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -3868,7 +3868,7 @@
         <v>100</v>
       </c>
       <c r="G10">
-        <v>33.64</v>
+        <v>35.48</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -3891,7 +3891,7 @@
         <v>100</v>
       </c>
       <c r="G11">
-        <v>36.04</v>
+        <v>38.32</v>
       </c>
     </row>
   </sheetData>
@@ -3957,7 +3957,7 @@
         <v>37</v>
       </c>
       <c r="F2">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G2" t="s">
         <v>38</v>
@@ -3983,7 +3983,7 @@
         <v>37</v>
       </c>
       <c r="F3">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="G3" t="s">
         <v>38</v>
@@ -4009,7 +4009,7 @@
         <v>37</v>
       </c>
       <c r="F4">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="G4" t="s">
         <v>38</v>
@@ -4035,7 +4035,7 @@
         <v>37</v>
       </c>
       <c r="F5">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="G5" t="s">
         <v>38</v>
@@ -4061,7 +4061,7 @@
         <v>37</v>
       </c>
       <c r="F6">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
         <v>38</v>
@@ -4087,7 +4087,7 @@
         <v>37</v>
       </c>
       <c r="F7">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
         <v>38</v>
@@ -4113,7 +4113,7 @@
         <v>37</v>
       </c>
       <c r="F8">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="G8" t="s">
         <v>38</v>
@@ -4139,7 +4139,7 @@
         <v>37</v>
       </c>
       <c r="F9">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="G9" t="s">
         <v>38</v>
@@ -4165,7 +4165,7 @@
         <v>37</v>
       </c>
       <c r="F10">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="G10" t="s">
         <v>38</v>
@@ -4191,7 +4191,7 @@
         <v>37</v>
       </c>
       <c r="F11">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="G11" t="s">
         <v>38</v>
@@ -4217,7 +4217,7 @@
         <v>37</v>
       </c>
       <c r="F12">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="G12" t="s">
         <v>38</v>
@@ -4243,7 +4243,7 @@
         <v>37</v>
       </c>
       <c r="F13">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="G13" t="s">
         <v>38</v>
@@ -4269,7 +4269,7 @@
         <v>37</v>
       </c>
       <c r="F14">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="G14" t="s">
         <v>38</v>
@@ -4295,7 +4295,7 @@
         <v>37</v>
       </c>
       <c r="F15">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="G15" t="s">
         <v>38</v>
@@ -4321,7 +4321,7 @@
         <v>37</v>
       </c>
       <c r="F16">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="G16" t="s">
         <v>38</v>
@@ -4347,7 +4347,7 @@
         <v>37</v>
       </c>
       <c r="F17">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="G17" t="s">
         <v>38</v>
@@ -4373,7 +4373,7 @@
         <v>37</v>
       </c>
       <c r="F18">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G18" t="s">
         <v>38</v>
@@ -4399,7 +4399,7 @@
         <v>37</v>
       </c>
       <c r="F19">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="G19" t="s">
         <v>38</v>
@@ -4425,7 +4425,7 @@
         <v>37</v>
       </c>
       <c r="F20">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="G20" t="s">
         <v>38</v>
@@ -4451,7 +4451,7 @@
         <v>37</v>
       </c>
       <c r="F21">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="G21" t="s">
         <v>38</v>
@@ -4477,7 +4477,7 @@
         <v>37</v>
       </c>
       <c r="F22">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="G22" t="s">
         <v>38</v>
@@ -4503,7 +4503,7 @@
         <v>37</v>
       </c>
       <c r="F23">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="G23" t="s">
         <v>38</v>
@@ -4529,7 +4529,7 @@
         <v>37</v>
       </c>
       <c r="F24">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="G24" t="s">
         <v>38</v>
@@ -4555,7 +4555,7 @@
         <v>37</v>
       </c>
       <c r="F25">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="G25" t="s">
         <v>38</v>
@@ -4581,7 +4581,7 @@
         <v>37</v>
       </c>
       <c r="F26">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G26" t="s">
         <v>38</v>
@@ -4607,7 +4607,7 @@
         <v>37</v>
       </c>
       <c r="F27">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="G27" t="s">
         <v>38</v>
@@ -4633,7 +4633,7 @@
         <v>37</v>
       </c>
       <c r="F28">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="G28" t="s">
         <v>38</v>
@@ -4659,7 +4659,7 @@
         <v>37</v>
       </c>
       <c r="F29">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="G29" t="s">
         <v>38</v>
@@ -4685,7 +4685,7 @@
         <v>37</v>
       </c>
       <c r="F30">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G30" t="s">
         <v>38</v>
@@ -4711,7 +4711,7 @@
         <v>37</v>
       </c>
       <c r="F31">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="G31" t="s">
         <v>38</v>
@@ -4737,7 +4737,7 @@
         <v>37</v>
       </c>
       <c r="F32">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="G32" t="s">
         <v>38</v>
@@ -4763,7 +4763,7 @@
         <v>37</v>
       </c>
       <c r="F33">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="G33" t="s">
         <v>38</v>
@@ -4789,7 +4789,7 @@
         <v>37</v>
       </c>
       <c r="F34">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G34" t="s">
         <v>38</v>
@@ -4815,7 +4815,7 @@
         <v>37</v>
       </c>
       <c r="F35">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="G35" t="s">
         <v>38</v>
@@ -4841,7 +4841,7 @@
         <v>37</v>
       </c>
       <c r="F36">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="G36" t="s">
         <v>38</v>
@@ -4867,7 +4867,7 @@
         <v>37</v>
       </c>
       <c r="F37">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="G37" t="s">
         <v>38</v>
@@ -4893,7 +4893,7 @@
         <v>37</v>
       </c>
       <c r="F38">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G38" t="s">
         <v>38</v>
@@ -4919,7 +4919,7 @@
         <v>37</v>
       </c>
       <c r="F39">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="G39" t="s">
         <v>38</v>
@@ -4945,7 +4945,7 @@
         <v>37</v>
       </c>
       <c r="F40">
-        <v>39</v>
+        <v>15</v>
       </c>
       <c r="G40" t="s">
         <v>38</v>
@@ -4971,7 +4971,7 @@
         <v>37</v>
       </c>
       <c r="F41">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G41" t="s">
         <v>38</v>
@@ -4997,7 +4997,7 @@
         <v>37</v>
       </c>
       <c r="F42">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="G42" t="s">
         <v>38</v>
@@ -5023,7 +5023,7 @@
         <v>37</v>
       </c>
       <c r="F43">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="G43" t="s">
         <v>38</v>
@@ -5049,7 +5049,7 @@
         <v>37</v>
       </c>
       <c r="F44">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="G44" t="s">
         <v>38</v>
@@ -5075,7 +5075,7 @@
         <v>37</v>
       </c>
       <c r="F45">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="G45" t="s">
         <v>38</v>
@@ -5101,7 +5101,7 @@
         <v>37</v>
       </c>
       <c r="F46">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="G46" t="s">
         <v>38</v>
@@ -5127,7 +5127,7 @@
         <v>37</v>
       </c>
       <c r="F47">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="G47" t="s">
         <v>38</v>
@@ -5153,7 +5153,7 @@
         <v>37</v>
       </c>
       <c r="F48">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="G48" t="s">
         <v>38</v>
@@ -5179,7 +5179,7 @@
         <v>37</v>
       </c>
       <c r="F49">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G49" t="s">
         <v>38</v>
@@ -5205,7 +5205,7 @@
         <v>37</v>
       </c>
       <c r="F50">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G50" t="s">
         <v>38</v>
@@ -5231,7 +5231,7 @@
         <v>37</v>
       </c>
       <c r="F51">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G51" t="s">
         <v>38</v>
@@ -5257,7 +5257,7 @@
         <v>37</v>
       </c>
       <c r="F52">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G52" t="s">
         <v>38</v>
@@ -5283,7 +5283,7 @@
         <v>37</v>
       </c>
       <c r="F53">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="G53" t="s">
         <v>38</v>
@@ -5309,7 +5309,7 @@
         <v>37</v>
       </c>
       <c r="F54">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G54" t="s">
         <v>38</v>
@@ -5335,7 +5335,7 @@
         <v>37</v>
       </c>
       <c r="F55">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="G55" t="s">
         <v>38</v>
@@ -5361,7 +5361,7 @@
         <v>37</v>
       </c>
       <c r="F56">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="G56" t="s">
         <v>38</v>
@@ -5387,7 +5387,7 @@
         <v>37</v>
       </c>
       <c r="F57">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="G57" t="s">
         <v>38</v>
@@ -5413,7 +5413,7 @@
         <v>37</v>
       </c>
       <c r="F58">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G58" t="s">
         <v>38</v>
@@ -5439,7 +5439,7 @@
         <v>37</v>
       </c>
       <c r="F59">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="G59" t="s">
         <v>38</v>
@@ -5465,7 +5465,7 @@
         <v>37</v>
       </c>
       <c r="F60">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="G60" t="s">
         <v>38</v>
@@ -5491,7 +5491,7 @@
         <v>37</v>
       </c>
       <c r="F61">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="G61" t="s">
         <v>38</v>
@@ -5517,7 +5517,7 @@
         <v>37</v>
       </c>
       <c r="F62">
-        <v>27</v>
+        <v>53</v>
       </c>
       <c r="G62" t="s">
         <v>38</v>
@@ -5543,7 +5543,7 @@
         <v>37</v>
       </c>
       <c r="F63">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="G63" t="s">
         <v>38</v>
@@ -5595,7 +5595,7 @@
         <v>37</v>
       </c>
       <c r="F65">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="G65" t="s">
         <v>38</v>
@@ -5621,7 +5621,7 @@
         <v>37</v>
       </c>
       <c r="F66">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="G66" t="s">
         <v>38</v>
@@ -5647,7 +5647,7 @@
         <v>37</v>
       </c>
       <c r="F67">
-        <v>28</v>
+        <v>51</v>
       </c>
       <c r="G67" t="s">
         <v>38</v>
@@ -5673,7 +5673,7 @@
         <v>37</v>
       </c>
       <c r="F68">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G68" t="s">
         <v>38</v>
@@ -5699,7 +5699,7 @@
         <v>37</v>
       </c>
       <c r="F69">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G69" t="s">
         <v>38</v>
@@ -5725,7 +5725,7 @@
         <v>37</v>
       </c>
       <c r="F70">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G70" t="s">
         <v>38</v>
@@ -5751,7 +5751,7 @@
         <v>37</v>
       </c>
       <c r="F71">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="G71" t="s">
         <v>38</v>
@@ -5777,7 +5777,7 @@
         <v>37</v>
       </c>
       <c r="F72">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="G72" t="s">
         <v>38</v>
@@ -5803,7 +5803,7 @@
         <v>37</v>
       </c>
       <c r="F73">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G73" t="s">
         <v>38</v>
@@ -5829,7 +5829,7 @@
         <v>37</v>
       </c>
       <c r="F74">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="G74" t="s">
         <v>38</v>
@@ -5855,7 +5855,7 @@
         <v>37</v>
       </c>
       <c r="F75">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="G75" t="s">
         <v>38</v>
@@ -5881,7 +5881,7 @@
         <v>37</v>
       </c>
       <c r="F76">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="G76" t="s">
         <v>38</v>
@@ -5907,7 +5907,7 @@
         <v>37</v>
       </c>
       <c r="F77">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G77" t="s">
         <v>38</v>
@@ -5933,7 +5933,7 @@
         <v>37</v>
       </c>
       <c r="F78">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="G78" t="s">
         <v>38</v>
@@ -5959,7 +5959,7 @@
         <v>37</v>
       </c>
       <c r="F79">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="G79" t="s">
         <v>38</v>
@@ -5985,7 +5985,7 @@
         <v>37</v>
       </c>
       <c r="F80">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G80" t="s">
         <v>38</v>
@@ -6011,7 +6011,7 @@
         <v>37</v>
       </c>
       <c r="F81">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G81" t="s">
         <v>38</v>
@@ -6037,7 +6037,7 @@
         <v>37</v>
       </c>
       <c r="F82">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="G82" t="s">
         <v>38</v>
@@ -6063,7 +6063,7 @@
         <v>37</v>
       </c>
       <c r="F83">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G83" t="s">
         <v>38</v>
@@ -6089,7 +6089,7 @@
         <v>37</v>
       </c>
       <c r="F84">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="G84" t="s">
         <v>38</v>
@@ -6115,7 +6115,7 @@
         <v>37</v>
       </c>
       <c r="F85">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="G85" t="s">
         <v>38</v>
@@ -6141,7 +6141,7 @@
         <v>37</v>
       </c>
       <c r="F86">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G86" t="s">
         <v>38</v>
@@ -6167,7 +6167,7 @@
         <v>37</v>
       </c>
       <c r="F87">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G87" t="s">
         <v>38</v>
@@ -6193,7 +6193,7 @@
         <v>37</v>
       </c>
       <c r="F88">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="G88" t="s">
         <v>38</v>
@@ -6219,7 +6219,7 @@
         <v>37</v>
       </c>
       <c r="F89">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="G89" t="s">
         <v>38</v>
@@ -6245,7 +6245,7 @@
         <v>37</v>
       </c>
       <c r="F90">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="G90" t="s">
         <v>38</v>
@@ -6271,7 +6271,7 @@
         <v>37</v>
       </c>
       <c r="F91">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="G91" t="s">
         <v>38</v>
@@ -6297,7 +6297,7 @@
         <v>37</v>
       </c>
       <c r="F92">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G92" t="s">
         <v>38</v>
@@ -6323,7 +6323,7 @@
         <v>37</v>
       </c>
       <c r="F93">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="G93" t="s">
         <v>38</v>
@@ -6349,7 +6349,7 @@
         <v>37</v>
       </c>
       <c r="F94">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="G94" t="s">
         <v>38</v>
@@ -6375,7 +6375,7 @@
         <v>37</v>
       </c>
       <c r="F95">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G95" t="s">
         <v>38</v>
@@ -6401,7 +6401,7 @@
         <v>37</v>
       </c>
       <c r="F96">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G96" t="s">
         <v>38</v>
@@ -6427,7 +6427,7 @@
         <v>37</v>
       </c>
       <c r="F97">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="G97" t="s">
         <v>38</v>
@@ -6453,7 +6453,7 @@
         <v>37</v>
       </c>
       <c r="F98">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="G98" t="s">
         <v>38</v>
@@ -6479,7 +6479,7 @@
         <v>37</v>
       </c>
       <c r="F99">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="G99" t="s">
         <v>38</v>
@@ -6505,7 +6505,7 @@
         <v>37</v>
       </c>
       <c r="F100">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="G100" t="s">
         <v>38</v>
@@ -6531,7 +6531,7 @@
         <v>37</v>
       </c>
       <c r="F101">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="G101" t="s">
         <v>38</v>
@@ -6583,7 +6583,7 @@
         <v>37</v>
       </c>
       <c r="F103">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G103" t="s">
         <v>38</v>
@@ -6609,7 +6609,7 @@
         <v>37</v>
       </c>
       <c r="F104">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G104" t="s">
         <v>38</v>
@@ -6635,7 +6635,7 @@
         <v>37</v>
       </c>
       <c r="F105">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="G105" t="s">
         <v>38</v>
@@ -6661,7 +6661,7 @@
         <v>37</v>
       </c>
       <c r="F106">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="G106" t="s">
         <v>38</v>
@@ -6687,7 +6687,7 @@
         <v>37</v>
       </c>
       <c r="F107">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G107" t="s">
         <v>38</v>
@@ -6713,7 +6713,7 @@
         <v>37</v>
       </c>
       <c r="F108">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="G108" t="s">
         <v>38</v>
@@ -6739,7 +6739,7 @@
         <v>37</v>
       </c>
       <c r="F109">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G109" t="s">
         <v>38</v>
@@ -6765,7 +6765,7 @@
         <v>37</v>
       </c>
       <c r="F110">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G110" t="s">
         <v>38</v>
@@ -6791,7 +6791,7 @@
         <v>37</v>
       </c>
       <c r="F111">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="G111" t="s">
         <v>38</v>
@@ -6817,7 +6817,7 @@
         <v>37</v>
       </c>
       <c r="F112">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G112" t="s">
         <v>38</v>
@@ -6843,7 +6843,7 @@
         <v>37</v>
       </c>
       <c r="F113">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="G113" t="s">
         <v>38</v>
@@ -6869,7 +6869,7 @@
         <v>37</v>
       </c>
       <c r="F114">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G114" t="s">
         <v>38</v>
@@ -6895,7 +6895,7 @@
         <v>37</v>
       </c>
       <c r="F115">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="G115" t="s">
         <v>38</v>
@@ -6921,7 +6921,7 @@
         <v>37</v>
       </c>
       <c r="F116">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="G116" t="s">
         <v>38</v>
@@ -6947,7 +6947,7 @@
         <v>37</v>
       </c>
       <c r="F117">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="G117" t="s">
         <v>38</v>
@@ -6973,7 +6973,7 @@
         <v>37</v>
       </c>
       <c r="F118">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G118" t="s">
         <v>38</v>
@@ -6999,7 +6999,7 @@
         <v>37</v>
       </c>
       <c r="F119">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="G119" t="s">
         <v>38</v>
@@ -7025,7 +7025,7 @@
         <v>37</v>
       </c>
       <c r="F120">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="G120" t="s">
         <v>38</v>
@@ -7051,7 +7051,7 @@
         <v>37</v>
       </c>
       <c r="F121">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="G121" t="s">
         <v>38</v>
@@ -7077,7 +7077,7 @@
         <v>37</v>
       </c>
       <c r="F122">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="G122" t="s">
         <v>38</v>
@@ -7103,7 +7103,7 @@
         <v>37</v>
       </c>
       <c r="F123">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="G123" t="s">
         <v>38</v>
@@ -7129,7 +7129,7 @@
         <v>37</v>
       </c>
       <c r="F124">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="G124" t="s">
         <v>38</v>
@@ -7155,7 +7155,7 @@
         <v>37</v>
       </c>
       <c r="F125">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G125" t="s">
         <v>38</v>
@@ -7181,7 +7181,7 @@
         <v>37</v>
       </c>
       <c r="F126">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G126" t="s">
         <v>38</v>
@@ -7207,7 +7207,7 @@
         <v>37</v>
       </c>
       <c r="F127">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="G127" t="s">
         <v>38</v>
@@ -7233,7 +7233,7 @@
         <v>37</v>
       </c>
       <c r="F128">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="G128" t="s">
         <v>38</v>
@@ -7259,7 +7259,7 @@
         <v>37</v>
       </c>
       <c r="F129">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="G129" t="s">
         <v>38</v>
@@ -7285,7 +7285,7 @@
         <v>37</v>
       </c>
       <c r="F130">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="G130" t="s">
         <v>38</v>
@@ -7311,7 +7311,7 @@
         <v>37</v>
       </c>
       <c r="F131">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="G131" t="s">
         <v>38</v>
@@ -7337,7 +7337,7 @@
         <v>37</v>
       </c>
       <c r="F132">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="G132" t="s">
         <v>38</v>
@@ -7363,7 +7363,7 @@
         <v>37</v>
       </c>
       <c r="F133">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="G133" t="s">
         <v>38</v>
@@ -7389,7 +7389,7 @@
         <v>37</v>
       </c>
       <c r="F134">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="G134" t="s">
         <v>38</v>
@@ -7415,7 +7415,7 @@
         <v>37</v>
       </c>
       <c r="F135">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="G135" t="s">
         <v>38</v>
@@ -7441,7 +7441,7 @@
         <v>37</v>
       </c>
       <c r="F136">
-        <v>19</v>
+        <v>41</v>
       </c>
       <c r="G136" t="s">
         <v>38</v>
@@ -7467,7 +7467,7 @@
         <v>37</v>
       </c>
       <c r="F137">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="G137" t="s">
         <v>38</v>
@@ -7493,7 +7493,7 @@
         <v>37</v>
       </c>
       <c r="F138">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="G138" t="s">
         <v>38</v>
@@ -7519,7 +7519,7 @@
         <v>37</v>
       </c>
       <c r="F139">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="G139" t="s">
         <v>38</v>
@@ -7545,7 +7545,7 @@
         <v>37</v>
       </c>
       <c r="F140">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="G140" t="s">
         <v>38</v>
@@ -7571,7 +7571,7 @@
         <v>37</v>
       </c>
       <c r="F141">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="G141" t="s">
         <v>38</v>
@@ -7597,7 +7597,7 @@
         <v>37</v>
       </c>
       <c r="F142">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G142" t="s">
         <v>38</v>
@@ -7623,7 +7623,7 @@
         <v>37</v>
       </c>
       <c r="F143">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="G143" t="s">
         <v>38</v>
@@ -7675,7 +7675,7 @@
         <v>37</v>
       </c>
       <c r="F145">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G145" t="s">
         <v>38</v>
@@ -7701,7 +7701,7 @@
         <v>37</v>
       </c>
       <c r="F146">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="G146" t="s">
         <v>38</v>
@@ -7727,7 +7727,7 @@
         <v>37</v>
       </c>
       <c r="F147">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="G147" t="s">
         <v>38</v>
@@ -7753,7 +7753,7 @@
         <v>37</v>
       </c>
       <c r="F148">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="G148" t="s">
         <v>38</v>
@@ -7779,7 +7779,7 @@
         <v>37</v>
       </c>
       <c r="F149">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="G149" t="s">
         <v>38</v>
@@ -7805,7 +7805,7 @@
         <v>37</v>
       </c>
       <c r="F150">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="G150" t="s">
         <v>38</v>
@@ -7831,7 +7831,7 @@
         <v>37</v>
       </c>
       <c r="F151">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G151" t="s">
         <v>38</v>
@@ -7857,7 +7857,7 @@
         <v>37</v>
       </c>
       <c r="F152">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G152" t="s">
         <v>38</v>
@@ -7883,7 +7883,7 @@
         <v>37</v>
       </c>
       <c r="F153">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="G153" t="s">
         <v>38</v>
@@ -7909,7 +7909,7 @@
         <v>37</v>
       </c>
       <c r="F154">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G154" t="s">
         <v>38</v>
@@ -7935,7 +7935,7 @@
         <v>37</v>
       </c>
       <c r="F155">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G155" t="s">
         <v>38</v>
@@ -7961,7 +7961,7 @@
         <v>37</v>
       </c>
       <c r="F156">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="G156" t="s">
         <v>38</v>
@@ -7987,7 +7987,7 @@
         <v>37</v>
       </c>
       <c r="F157">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="G157" t="s">
         <v>38</v>
@@ -8013,7 +8013,7 @@
         <v>37</v>
       </c>
       <c r="F158">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="G158" t="s">
         <v>38</v>
@@ -8039,7 +8039,7 @@
         <v>37</v>
       </c>
       <c r="F159">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="G159" t="s">
         <v>38</v>
@@ -8065,7 +8065,7 @@
         <v>37</v>
       </c>
       <c r="F160">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="G160" t="s">
         <v>38</v>
@@ -8117,7 +8117,7 @@
         <v>37</v>
       </c>
       <c r="F162">
-        <v>54</v>
+        <v>39</v>
       </c>
       <c r="G162" t="s">
         <v>38</v>
@@ -8143,7 +8143,7 @@
         <v>37</v>
       </c>
       <c r="F163">
-        <v>25</v>
+        <v>47</v>
       </c>
       <c r="G163" t="s">
         <v>38</v>
@@ -8169,7 +8169,7 @@
         <v>37</v>
       </c>
       <c r="F164">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="G164" t="s">
         <v>38</v>
@@ -8195,7 +8195,7 @@
         <v>37</v>
       </c>
       <c r="F165">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="G165" t="s">
         <v>38</v>
@@ -8221,7 +8221,7 @@
         <v>37</v>
       </c>
       <c r="F166">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="G166" t="s">
         <v>38</v>
@@ -8247,7 +8247,7 @@
         <v>37</v>
       </c>
       <c r="F167">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G167" t="s">
         <v>38</v>
@@ -8273,7 +8273,7 @@
         <v>37</v>
       </c>
       <c r="F168">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="G168" t="s">
         <v>38</v>
@@ -8299,7 +8299,7 @@
         <v>37</v>
       </c>
       <c r="F169">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="G169" t="s">
         <v>38</v>
@@ -8325,7 +8325,7 @@
         <v>37</v>
       </c>
       <c r="F170">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="G170" t="s">
         <v>38</v>
@@ -8351,7 +8351,7 @@
         <v>37</v>
       </c>
       <c r="F171">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G171" t="s">
         <v>38</v>
@@ -8377,7 +8377,7 @@
         <v>37</v>
       </c>
       <c r="F172">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="G172" t="s">
         <v>38</v>
@@ -8403,7 +8403,7 @@
         <v>37</v>
       </c>
       <c r="F173">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="G173" t="s">
         <v>38</v>
@@ -8429,7 +8429,7 @@
         <v>37</v>
       </c>
       <c r="F174">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G174" t="s">
         <v>38</v>
@@ -8455,7 +8455,7 @@
         <v>37</v>
       </c>
       <c r="F175">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G175" t="s">
         <v>38</v>
@@ -8481,7 +8481,7 @@
         <v>37</v>
       </c>
       <c r="F176">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G176" t="s">
         <v>38</v>
@@ -8507,7 +8507,7 @@
         <v>37</v>
       </c>
       <c r="F177">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="G177" t="s">
         <v>38</v>
@@ -8533,7 +8533,7 @@
         <v>37</v>
       </c>
       <c r="F178">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="G178" t="s">
         <v>38</v>
@@ -8559,7 +8559,7 @@
         <v>37</v>
       </c>
       <c r="F179">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G179" t="s">
         <v>38</v>
@@ -8585,7 +8585,7 @@
         <v>37</v>
       </c>
       <c r="F180">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="G180" t="s">
         <v>38</v>
@@ -8611,7 +8611,7 @@
         <v>37</v>
       </c>
       <c r="F181">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="G181" t="s">
         <v>38</v>
@@ -8637,7 +8637,7 @@
         <v>37</v>
       </c>
       <c r="F182">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G182" t="s">
         <v>38</v>
@@ -8663,7 +8663,7 @@
         <v>37</v>
       </c>
       <c r="F183">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="G183" t="s">
         <v>38</v>
@@ -8689,7 +8689,7 @@
         <v>37</v>
       </c>
       <c r="F184">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G184" t="s">
         <v>38</v>
@@ -8715,7 +8715,7 @@
         <v>37</v>
       </c>
       <c r="F185">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="G185" t="s">
         <v>38</v>
@@ -8741,7 +8741,7 @@
         <v>37</v>
       </c>
       <c r="F186">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="G186" t="s">
         <v>38</v>
@@ -8767,7 +8767,7 @@
         <v>37</v>
       </c>
       <c r="F187">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="G187" t="s">
         <v>38</v>
@@ -8793,7 +8793,7 @@
         <v>37</v>
       </c>
       <c r="F188">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="G188" t="s">
         <v>38</v>
@@ -8845,7 +8845,7 @@
         <v>37</v>
       </c>
       <c r="F190">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G190" t="s">
         <v>38</v>
@@ -8871,7 +8871,7 @@
         <v>37</v>
       </c>
       <c r="F191">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G191" t="s">
         <v>38</v>
@@ -8897,7 +8897,7 @@
         <v>37</v>
       </c>
       <c r="F192">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="G192" t="s">
         <v>38</v>
@@ -8923,7 +8923,7 @@
         <v>37</v>
       </c>
       <c r="F193">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="G193" t="s">
         <v>38</v>
@@ -8949,7 +8949,7 @@
         <v>37</v>
       </c>
       <c r="F194">
-        <v>28</v>
+        <v>54</v>
       </c>
       <c r="G194" t="s">
         <v>38</v>
@@ -8975,7 +8975,7 @@
         <v>37</v>
       </c>
       <c r="F195">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="G195" t="s">
         <v>38</v>
@@ -9001,7 +9001,7 @@
         <v>37</v>
       </c>
       <c r="F196">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="G196" t="s">
         <v>38</v>
@@ -9027,7 +9027,7 @@
         <v>37</v>
       </c>
       <c r="F197">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G197" t="s">
         <v>38</v>
@@ -9053,7 +9053,7 @@
         <v>37</v>
       </c>
       <c r="F198">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="G198" t="s">
         <v>38</v>
@@ -9079,7 +9079,7 @@
         <v>37</v>
       </c>
       <c r="F199">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="G199" t="s">
         <v>38</v>
@@ -9105,7 +9105,7 @@
         <v>37</v>
       </c>
       <c r="F200">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="G200" t="s">
         <v>38</v>
@@ -9131,7 +9131,7 @@
         <v>37</v>
       </c>
       <c r="F201">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G201" t="s">
         <v>38</v>
@@ -9157,7 +9157,7 @@
         <v>37</v>
       </c>
       <c r="F202">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G202" t="s">
         <v>38</v>
@@ -9183,7 +9183,7 @@
         <v>37</v>
       </c>
       <c r="F203">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G203" t="s">
         <v>38</v>
@@ -9209,7 +9209,7 @@
         <v>37</v>
       </c>
       <c r="F204">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="G204" t="s">
         <v>38</v>
@@ -9235,7 +9235,7 @@
         <v>37</v>
       </c>
       <c r="F205">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="G205" t="s">
         <v>38</v>
@@ -9261,7 +9261,7 @@
         <v>37</v>
       </c>
       <c r="F206">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G206" t="s">
         <v>38</v>
@@ -9287,7 +9287,7 @@
         <v>37</v>
       </c>
       <c r="F207">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="G207" t="s">
         <v>38</v>
@@ -9313,7 +9313,7 @@
         <v>37</v>
       </c>
       <c r="F208">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="G208" t="s">
         <v>38</v>
@@ -9339,7 +9339,7 @@
         <v>37</v>
       </c>
       <c r="F209">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="G209" t="s">
         <v>38</v>
@@ -9365,7 +9365,7 @@
         <v>37</v>
       </c>
       <c r="F210">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="G210" t="s">
         <v>38</v>
@@ -9391,7 +9391,7 @@
         <v>37</v>
       </c>
       <c r="F211">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="G211" t="s">
         <v>38</v>
@@ -9417,7 +9417,7 @@
         <v>37</v>
       </c>
       <c r="F212">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="G212" t="s">
         <v>38</v>
@@ -9443,7 +9443,7 @@
         <v>37</v>
       </c>
       <c r="F213">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="G213" t="s">
         <v>38</v>
@@ -9469,7 +9469,7 @@
         <v>37</v>
       </c>
       <c r="F214">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="G214" t="s">
         <v>38</v>
@@ -9495,7 +9495,7 @@
         <v>37</v>
       </c>
       <c r="F215">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="G215" t="s">
         <v>38</v>
@@ -9521,7 +9521,7 @@
         <v>37</v>
       </c>
       <c r="F216">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G216" t="s">
         <v>38</v>
@@ -9547,7 +9547,7 @@
         <v>37</v>
       </c>
       <c r="F217">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="G217" t="s">
         <v>38</v>
@@ -9573,7 +9573,7 @@
         <v>37</v>
       </c>
       <c r="F218">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="G218" t="s">
         <v>38</v>
@@ -9599,7 +9599,7 @@
         <v>37</v>
       </c>
       <c r="F219">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G219" t="s">
         <v>38</v>
@@ -9625,7 +9625,7 @@
         <v>37</v>
       </c>
       <c r="F220">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="G220" t="s">
         <v>38</v>
@@ -9651,7 +9651,7 @@
         <v>37</v>
       </c>
       <c r="F221">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="G221" t="s">
         <v>38</v>
@@ -9677,7 +9677,7 @@
         <v>37</v>
       </c>
       <c r="F222">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="G222" t="s">
         <v>38</v>
@@ -9703,7 +9703,7 @@
         <v>37</v>
       </c>
       <c r="F223">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="G223" t="s">
         <v>38</v>
@@ -9729,7 +9729,7 @@
         <v>37</v>
       </c>
       <c r="F224">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G224" t="s">
         <v>38</v>
@@ -9755,7 +9755,7 @@
         <v>37</v>
       </c>
       <c r="F225">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="G225" t="s">
         <v>38</v>
@@ -9781,7 +9781,7 @@
         <v>37</v>
       </c>
       <c r="F226">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="G226" t="s">
         <v>38</v>
@@ -9807,7 +9807,7 @@
         <v>37</v>
       </c>
       <c r="F227">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="G227" t="s">
         <v>38</v>
@@ -9833,7 +9833,7 @@
         <v>37</v>
       </c>
       <c r="F228">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="G228" t="s">
         <v>38</v>
@@ -9859,7 +9859,7 @@
         <v>37</v>
       </c>
       <c r="F229">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="G229" t="s">
         <v>38</v>
@@ -9885,7 +9885,7 @@
         <v>37</v>
       </c>
       <c r="F230">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="G230" t="s">
         <v>38</v>
@@ -9911,7 +9911,7 @@
         <v>37</v>
       </c>
       <c r="F231">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="G231" t="s">
         <v>38</v>
@@ -9937,7 +9937,7 @@
         <v>37</v>
       </c>
       <c r="F232">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G232" t="s">
         <v>38</v>
@@ -9963,7 +9963,7 @@
         <v>37</v>
       </c>
       <c r="F233">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="G233" t="s">
         <v>38</v>
@@ -9989,7 +9989,7 @@
         <v>37</v>
       </c>
       <c r="F234">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="G234" t="s">
         <v>38</v>
@@ -10015,7 +10015,7 @@
         <v>37</v>
       </c>
       <c r="F235">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="G235" t="s">
         <v>38</v>
@@ -10041,7 +10041,7 @@
         <v>37</v>
       </c>
       <c r="F236">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G236" t="s">
         <v>38</v>
@@ -10067,7 +10067,7 @@
         <v>37</v>
       </c>
       <c r="F237">
-        <v>51</v>
+        <v>33</v>
       </c>
       <c r="G237" t="s">
         <v>38</v>
@@ -10093,7 +10093,7 @@
         <v>37</v>
       </c>
       <c r="F238">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G238" t="s">
         <v>38</v>
@@ -10119,7 +10119,7 @@
         <v>37</v>
       </c>
       <c r="F239">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="G239" t="s">
         <v>38</v>
@@ -10145,7 +10145,7 @@
         <v>37</v>
       </c>
       <c r="F240">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="G240" t="s">
         <v>38</v>
@@ -10171,7 +10171,7 @@
         <v>37</v>
       </c>
       <c r="F241">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="G241" t="s">
         <v>38</v>
@@ -10197,7 +10197,7 @@
         <v>37</v>
       </c>
       <c r="F242">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="G242" t="s">
         <v>38</v>
@@ -10223,7 +10223,7 @@
         <v>37</v>
       </c>
       <c r="F243">
-        <v>53</v>
+        <v>20</v>
       </c>
       <c r="G243" t="s">
         <v>38</v>
@@ -10249,7 +10249,7 @@
         <v>37</v>
       </c>
       <c r="F244">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="G244" t="s">
         <v>38</v>
@@ -10275,7 +10275,7 @@
         <v>37</v>
       </c>
       <c r="F245">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="G245" t="s">
         <v>38</v>
@@ -10301,7 +10301,7 @@
         <v>37</v>
       </c>
       <c r="F246">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="G246" t="s">
         <v>38</v>
@@ -10327,7 +10327,7 @@
         <v>37</v>
       </c>
       <c r="F247">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="G247" t="s">
         <v>38</v>
@@ -10353,7 +10353,7 @@
         <v>37</v>
       </c>
       <c r="F248">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G248" t="s">
         <v>38</v>
@@ -10379,7 +10379,7 @@
         <v>37</v>
       </c>
       <c r="F249">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G249" t="s">
         <v>38</v>
@@ -10405,7 +10405,7 @@
         <v>37</v>
       </c>
       <c r="F250">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G250" t="s">
         <v>38</v>
@@ -10431,7 +10431,7 @@
         <v>37</v>
       </c>
       <c r="F251">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G251" t="s">
         <v>38</v>
@@ -10457,7 +10457,7 @@
         <v>37</v>
       </c>
       <c r="F252">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="G252" t="s">
         <v>38</v>
@@ -10483,7 +10483,7 @@
         <v>37</v>
       </c>
       <c r="F253">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="G253" t="s">
         <v>38</v>
@@ -10509,7 +10509,7 @@
         <v>37</v>
       </c>
       <c r="F254">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G254" t="s">
         <v>38</v>
@@ -10535,7 +10535,7 @@
         <v>37</v>
       </c>
       <c r="F255">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="G255" t="s">
         <v>38</v>
@@ -10561,7 +10561,7 @@
         <v>37</v>
       </c>
       <c r="F256">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="G256" t="s">
         <v>38</v>
@@ -10587,7 +10587,7 @@
         <v>37</v>
       </c>
       <c r="F257">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="G257" t="s">
         <v>38</v>
@@ -10613,7 +10613,7 @@
         <v>37</v>
       </c>
       <c r="F258">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="G258" t="s">
         <v>38</v>
@@ -10639,7 +10639,7 @@
         <v>37</v>
       </c>
       <c r="F259">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="G259" t="s">
         <v>38</v>
@@ -10665,7 +10665,7 @@
         <v>37</v>
       </c>
       <c r="F260">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="G260" t="s">
         <v>38</v>
@@ -10691,7 +10691,7 @@
         <v>37</v>
       </c>
       <c r="F261">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G261" t="s">
         <v>38</v>
@@ -10717,7 +10717,7 @@
         <v>37</v>
       </c>
       <c r="F262">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="G262" t="s">
         <v>38</v>
@@ -10743,7 +10743,7 @@
         <v>37</v>
       </c>
       <c r="F263">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="G263" t="s">
         <v>38</v>
@@ -10769,7 +10769,7 @@
         <v>37</v>
       </c>
       <c r="F264">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G264" t="s">
         <v>38</v>
@@ -10795,7 +10795,7 @@
         <v>37</v>
       </c>
       <c r="F265">
-        <v>24</v>
+        <v>32</v>
       </c>
       <c r="G265" t="s">
         <v>38</v>
@@ -10821,7 +10821,7 @@
         <v>37</v>
       </c>
       <c r="F266">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="G266" t="s">
         <v>38</v>
@@ -10847,7 +10847,7 @@
         <v>37</v>
       </c>
       <c r="F267">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="G267" t="s">
         <v>38</v>
@@ -10873,7 +10873,7 @@
         <v>37</v>
       </c>
       <c r="F268">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="G268" t="s">
         <v>38</v>
@@ -10899,7 +10899,7 @@
         <v>37</v>
       </c>
       <c r="F269">
-        <v>26</v>
+        <v>51</v>
       </c>
       <c r="G269" t="s">
         <v>38</v>
@@ -10925,7 +10925,7 @@
         <v>37</v>
       </c>
       <c r="F270">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="G270" t="s">
         <v>38</v>
@@ -10951,7 +10951,7 @@
         <v>37</v>
       </c>
       <c r="F271">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="G271" t="s">
         <v>38</v>
@@ -10977,7 +10977,7 @@
         <v>37</v>
       </c>
       <c r="F272">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G272" t="s">
         <v>38</v>
@@ -11003,7 +11003,7 @@
         <v>37</v>
       </c>
       <c r="F273">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G273" t="s">
         <v>38</v>
@@ -11029,7 +11029,7 @@
         <v>37</v>
       </c>
       <c r="F274">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="G274" t="s">
         <v>38</v>
@@ -11055,7 +11055,7 @@
         <v>37</v>
       </c>
       <c r="F275">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G275" t="s">
         <v>38</v>
@@ -11081,7 +11081,7 @@
         <v>37</v>
       </c>
       <c r="F276">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G276" t="s">
         <v>38</v>
@@ -11107,7 +11107,7 @@
         <v>37</v>
       </c>
       <c r="F277">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="G277" t="s">
         <v>38</v>
@@ -11133,7 +11133,7 @@
         <v>37</v>
       </c>
       <c r="F278">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="G278" t="s">
         <v>38</v>
@@ -11185,7 +11185,7 @@
         <v>37</v>
       </c>
       <c r="F280">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="G280" t="s">
         <v>38</v>
@@ -11211,7 +11211,7 @@
         <v>37</v>
       </c>
       <c r="F281">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="G281" t="s">
         <v>38</v>
@@ -11237,7 +11237,7 @@
         <v>37</v>
       </c>
       <c r="F282">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="G282" t="s">
         <v>38</v>
@@ -11263,7 +11263,7 @@
         <v>37</v>
       </c>
       <c r="F283">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="G283" t="s">
         <v>38</v>
@@ -11289,7 +11289,7 @@
         <v>37</v>
       </c>
       <c r="F284">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="G284" t="s">
         <v>38</v>
@@ -11315,7 +11315,7 @@
         <v>37</v>
       </c>
       <c r="F285">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="G285" t="s">
         <v>38</v>
@@ -11341,7 +11341,7 @@
         <v>37</v>
       </c>
       <c r="F286">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="G286" t="s">
         <v>38</v>
@@ -11367,7 +11367,7 @@
         <v>37</v>
       </c>
       <c r="F287">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G287" t="s">
         <v>38</v>
@@ -11393,7 +11393,7 @@
         <v>37</v>
       </c>
       <c r="F288">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="G288" t="s">
         <v>38</v>
@@ -11419,7 +11419,7 @@
         <v>37</v>
       </c>
       <c r="F289">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G289" t="s">
         <v>38</v>
@@ -11445,7 +11445,7 @@
         <v>37</v>
       </c>
       <c r="F290">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="G290" t="s">
         <v>38</v>
@@ -11471,7 +11471,7 @@
         <v>37</v>
       </c>
       <c r="F291">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="G291" t="s">
         <v>38</v>
@@ -11497,7 +11497,7 @@
         <v>37</v>
       </c>
       <c r="F292">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="G292" t="s">
         <v>38</v>
@@ -11523,7 +11523,7 @@
         <v>37</v>
       </c>
       <c r="F293">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="G293" t="s">
         <v>38</v>
@@ -11549,7 +11549,7 @@
         <v>37</v>
       </c>
       <c r="F294">
-        <v>27</v>
+        <v>52</v>
       </c>
       <c r="G294" t="s">
         <v>38</v>
@@ -11601,7 +11601,7 @@
         <v>37</v>
       </c>
       <c r="F296">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="G296" t="s">
         <v>38</v>
@@ -11627,7 +11627,7 @@
         <v>37</v>
       </c>
       <c r="F297">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="G297" t="s">
         <v>38</v>
@@ -11653,7 +11653,7 @@
         <v>37</v>
       </c>
       <c r="F298">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="G298" t="s">
         <v>38</v>
@@ -11705,7 +11705,7 @@
         <v>37</v>
       </c>
       <c r="F300">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G300" t="s">
         <v>38</v>
@@ -11731,7 +11731,7 @@
         <v>37</v>
       </c>
       <c r="F301">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="G301" t="s">
         <v>38</v>
@@ -11757,7 +11757,7 @@
         <v>37</v>
       </c>
       <c r="F302">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="G302" t="s">
         <v>38</v>
@@ -11783,7 +11783,7 @@
         <v>37</v>
       </c>
       <c r="F303">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G303" t="s">
         <v>38</v>
@@ -11809,7 +11809,7 @@
         <v>37</v>
       </c>
       <c r="F304">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="G304" t="s">
         <v>38</v>
@@ -11835,7 +11835,7 @@
         <v>37</v>
       </c>
       <c r="F305">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G305" t="s">
         <v>38</v>
@@ -11861,7 +11861,7 @@
         <v>37</v>
       </c>
       <c r="F306">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="G306" t="s">
         <v>38</v>
@@ -11887,7 +11887,7 @@
         <v>37</v>
       </c>
       <c r="F307">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="G307" t="s">
         <v>38</v>
@@ -11913,7 +11913,7 @@
         <v>37</v>
       </c>
       <c r="F308">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G308" t="s">
         <v>38</v>
@@ -11991,7 +11991,7 @@
         <v>37</v>
       </c>
       <c r="F311">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="G311" t="s">
         <v>38</v>
@@ -12017,7 +12017,7 @@
         <v>37</v>
       </c>
       <c r="F312">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="G312" t="s">
         <v>38</v>
@@ -12043,7 +12043,7 @@
         <v>37</v>
       </c>
       <c r="F313">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="G313" t="s">
         <v>38</v>
@@ -12069,7 +12069,7 @@
         <v>37</v>
       </c>
       <c r="F314">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G314" t="s">
         <v>38</v>
@@ -12095,7 +12095,7 @@
         <v>37</v>
       </c>
       <c r="F315">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="G315" t="s">
         <v>38</v>
@@ -12121,7 +12121,7 @@
         <v>37</v>
       </c>
       <c r="F316">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="G316" t="s">
         <v>38</v>
@@ -12147,7 +12147,7 @@
         <v>37</v>
       </c>
       <c r="F317">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="G317" t="s">
         <v>38</v>
@@ -12173,7 +12173,7 @@
         <v>37</v>
       </c>
       <c r="F318">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="G318" t="s">
         <v>38</v>
@@ -12199,7 +12199,7 @@
         <v>37</v>
       </c>
       <c r="F319">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G319" t="s">
         <v>38</v>
@@ -12225,7 +12225,7 @@
         <v>37</v>
       </c>
       <c r="F320">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="G320" t="s">
         <v>38</v>
@@ -12251,7 +12251,7 @@
         <v>37</v>
       </c>
       <c r="F321">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G321" t="s">
         <v>38</v>
@@ -12277,7 +12277,7 @@
         <v>37</v>
       </c>
       <c r="F322">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="G322" t="s">
         <v>38</v>
@@ -12303,7 +12303,7 @@
         <v>37</v>
       </c>
       <c r="F323">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="G323" t="s">
         <v>38</v>
@@ -12329,7 +12329,7 @@
         <v>37</v>
       </c>
       <c r="F324">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="G324" t="s">
         <v>38</v>
@@ -12355,7 +12355,7 @@
         <v>37</v>
       </c>
       <c r="F325">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G325" t="s">
         <v>38</v>
@@ -12381,7 +12381,7 @@
         <v>37</v>
       </c>
       <c r="F326">
-        <v>24</v>
+        <v>49</v>
       </c>
       <c r="G326" t="s">
         <v>38</v>
@@ -12407,7 +12407,7 @@
         <v>37</v>
       </c>
       <c r="F327">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="G327" t="s">
         <v>38</v>
@@ -12433,7 +12433,7 @@
         <v>37</v>
       </c>
       <c r="F328">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="G328" t="s">
         <v>38</v>
@@ -12459,7 +12459,7 @@
         <v>37</v>
       </c>
       <c r="F329">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="G329" t="s">
         <v>38</v>
@@ -12485,7 +12485,7 @@
         <v>37</v>
       </c>
       <c r="F330">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G330" t="s">
         <v>38</v>
@@ -12511,7 +12511,7 @@
         <v>37</v>
       </c>
       <c r="F331">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="G331" t="s">
         <v>38</v>
@@ -12537,7 +12537,7 @@
         <v>37</v>
       </c>
       <c r="F332">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="G332" t="s">
         <v>38</v>
@@ -12563,7 +12563,7 @@
         <v>37</v>
       </c>
       <c r="F333">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="G333" t="s">
         <v>38</v>
@@ -12589,7 +12589,7 @@
         <v>37</v>
       </c>
       <c r="F334">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="G334" t="s">
         <v>38</v>
@@ -12615,7 +12615,7 @@
         <v>37</v>
       </c>
       <c r="F335">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G335" t="s">
         <v>38</v>
@@ -12641,7 +12641,7 @@
         <v>37</v>
       </c>
       <c r="F336">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G336" t="s">
         <v>38</v>
@@ -12667,7 +12667,7 @@
         <v>37</v>
       </c>
       <c r="F337">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="G337" t="s">
         <v>38</v>
@@ -12693,7 +12693,7 @@
         <v>37</v>
       </c>
       <c r="F338">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="G338" t="s">
         <v>38</v>
@@ -12719,7 +12719,7 @@
         <v>37</v>
       </c>
       <c r="F339">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="G339" t="s">
         <v>38</v>
@@ -12745,7 +12745,7 @@
         <v>37</v>
       </c>
       <c r="F340">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="G340" t="s">
         <v>38</v>
@@ -12771,7 +12771,7 @@
         <v>37</v>
       </c>
       <c r="F341">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="G341" t="s">
         <v>38</v>
@@ -12797,7 +12797,7 @@
         <v>37</v>
       </c>
       <c r="F342">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="G342" t="s">
         <v>38</v>
@@ -12823,7 +12823,7 @@
         <v>37</v>
       </c>
       <c r="F343">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="G343" t="s">
         <v>38</v>
@@ -12849,7 +12849,7 @@
         <v>37</v>
       </c>
       <c r="F344">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="G344" t="s">
         <v>38</v>
@@ -12875,7 +12875,7 @@
         <v>37</v>
       </c>
       <c r="F345">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G345" t="s">
         <v>38</v>
@@ -12901,7 +12901,7 @@
         <v>37</v>
       </c>
       <c r="F346">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G346" t="s">
         <v>38</v>
@@ -12927,7 +12927,7 @@
         <v>37</v>
       </c>
       <c r="F347">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="G347" t="s">
         <v>38</v>
@@ -12953,7 +12953,7 @@
         <v>37</v>
       </c>
       <c r="F348">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="G348" t="s">
         <v>38</v>
@@ -12979,7 +12979,7 @@
         <v>37</v>
       </c>
       <c r="F349">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="G349" t="s">
         <v>38</v>
@@ -13005,7 +13005,7 @@
         <v>37</v>
       </c>
       <c r="F350">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="G350" t="s">
         <v>38</v>
@@ -13031,7 +13031,7 @@
         <v>37</v>
       </c>
       <c r="F351">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="G351" t="s">
         <v>38</v>
@@ -13057,7 +13057,7 @@
         <v>37</v>
       </c>
       <c r="F352">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G352" t="s">
         <v>38</v>
@@ -13083,7 +13083,7 @@
         <v>37</v>
       </c>
       <c r="F353">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="G353" t="s">
         <v>38</v>
@@ -13109,7 +13109,7 @@
         <v>37</v>
       </c>
       <c r="F354">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="G354" t="s">
         <v>38</v>
@@ -13135,7 +13135,7 @@
         <v>37</v>
       </c>
       <c r="F355">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="G355" t="s">
         <v>38</v>
@@ -13161,7 +13161,7 @@
         <v>37</v>
       </c>
       <c r="F356">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G356" t="s">
         <v>38</v>
@@ -13187,7 +13187,7 @@
         <v>37</v>
       </c>
       <c r="F357">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G357" t="s">
         <v>38</v>
@@ -13213,7 +13213,7 @@
         <v>37</v>
       </c>
       <c r="F358">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="G358" t="s">
         <v>38</v>
@@ -13239,7 +13239,7 @@
         <v>37</v>
       </c>
       <c r="F359">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="G359" t="s">
         <v>38</v>
@@ -13265,7 +13265,7 @@
         <v>37</v>
       </c>
       <c r="F360">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="G360" t="s">
         <v>38</v>
@@ -13291,7 +13291,7 @@
         <v>37</v>
       </c>
       <c r="F361">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="G361" t="s">
         <v>38</v>
@@ -13317,7 +13317,7 @@
         <v>37</v>
       </c>
       <c r="F362">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="G362" t="s">
         <v>38</v>
@@ -13343,7 +13343,7 @@
         <v>37</v>
       </c>
       <c r="F363">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="G363" t="s">
         <v>38</v>
@@ -13369,7 +13369,7 @@
         <v>37</v>
       </c>
       <c r="F364">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="G364" t="s">
         <v>38</v>
@@ -13395,7 +13395,7 @@
         <v>37</v>
       </c>
       <c r="F365">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G365" t="s">
         <v>38</v>
@@ -13421,7 +13421,7 @@
         <v>37</v>
       </c>
       <c r="F366">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="G366" t="s">
         <v>38</v>
@@ -13447,7 +13447,7 @@
         <v>37</v>
       </c>
       <c r="F367">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="G367" t="s">
         <v>38</v>
@@ -13473,7 +13473,7 @@
         <v>37</v>
       </c>
       <c r="F368">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="G368" t="s">
         <v>38</v>
@@ -13499,7 +13499,7 @@
         <v>37</v>
       </c>
       <c r="F369">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="G369" t="s">
         <v>38</v>
@@ -13525,7 +13525,7 @@
         <v>37</v>
       </c>
       <c r="F370">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G370" t="s">
         <v>38</v>
@@ -13551,7 +13551,7 @@
         <v>37</v>
       </c>
       <c r="F371">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G371" t="s">
         <v>38</v>
@@ -13577,7 +13577,7 @@
         <v>37</v>
       </c>
       <c r="F372">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="G372" t="s">
         <v>38</v>
@@ -13603,7 +13603,7 @@
         <v>37</v>
       </c>
       <c r="F373">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="G373" t="s">
         <v>38</v>
@@ -13629,7 +13629,7 @@
         <v>37</v>
       </c>
       <c r="F374">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="G374" t="s">
         <v>38</v>
@@ -13655,7 +13655,7 @@
         <v>37</v>
       </c>
       <c r="F375">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="G375" t="s">
         <v>38</v>
@@ -13681,7 +13681,7 @@
         <v>37</v>
       </c>
       <c r="F376">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="G376" t="s">
         <v>38</v>
@@ -13707,7 +13707,7 @@
         <v>37</v>
       </c>
       <c r="F377">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G377" t="s">
         <v>38</v>
@@ -13733,7 +13733,7 @@
         <v>37</v>
       </c>
       <c r="F378">
-        <v>23</v>
+        <v>44</v>
       </c>
       <c r="G378" t="s">
         <v>38</v>
@@ -13759,7 +13759,7 @@
         <v>37</v>
       </c>
       <c r="F379">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="G379" t="s">
         <v>38</v>
@@ -13811,7 +13811,7 @@
         <v>37</v>
       </c>
       <c r="F381">
-        <v>19</v>
+        <v>54</v>
       </c>
       <c r="G381" t="s">
         <v>38</v>
@@ -13837,7 +13837,7 @@
         <v>37</v>
       </c>
       <c r="F382">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G382" t="s">
         <v>38</v>
@@ -13863,7 +13863,7 @@
         <v>37</v>
       </c>
       <c r="F383">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="G383" t="s">
         <v>38</v>
@@ -13889,7 +13889,7 @@
         <v>37</v>
       </c>
       <c r="F384">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="G384" t="s">
         <v>38</v>
@@ -13915,7 +13915,7 @@
         <v>37</v>
       </c>
       <c r="F385">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="G385" t="s">
         <v>38</v>
@@ -13941,7 +13941,7 @@
         <v>37</v>
       </c>
       <c r="F386">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G386" t="s">
         <v>38</v>
@@ -13967,7 +13967,7 @@
         <v>37</v>
       </c>
       <c r="F387">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G387" t="s">
         <v>38</v>
@@ -13993,7 +13993,7 @@
         <v>37</v>
       </c>
       <c r="F388">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="G388" t="s">
         <v>38</v>
@@ -14019,7 +14019,7 @@
         <v>37</v>
       </c>
       <c r="F389">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G389" t="s">
         <v>38</v>
@@ -14045,7 +14045,7 @@
         <v>37</v>
       </c>
       <c r="F390">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G390" t="s">
         <v>38</v>
@@ -14071,7 +14071,7 @@
         <v>37</v>
       </c>
       <c r="F391">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="G391" t="s">
         <v>38</v>
@@ -14097,7 +14097,7 @@
         <v>37</v>
       </c>
       <c r="F392">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G392" t="s">
         <v>38</v>
@@ -14123,7 +14123,7 @@
         <v>37</v>
       </c>
       <c r="F393">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="G393" t="s">
         <v>38</v>
@@ -14149,7 +14149,7 @@
         <v>37</v>
       </c>
       <c r="F394">
-        <v>43</v>
+        <v>15</v>
       </c>
       <c r="G394" t="s">
         <v>38</v>
@@ -14175,7 +14175,7 @@
         <v>37</v>
       </c>
       <c r="F395">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="G395" t="s">
         <v>38</v>
@@ -14201,7 +14201,7 @@
         <v>37</v>
       </c>
       <c r="F396">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G396" t="s">
         <v>38</v>
@@ -14227,7 +14227,7 @@
         <v>37</v>
       </c>
       <c r="F397">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G397" t="s">
         <v>38</v>
@@ -14253,7 +14253,7 @@
         <v>37</v>
       </c>
       <c r="F398">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G398" t="s">
         <v>38</v>
@@ -14279,7 +14279,7 @@
         <v>37</v>
       </c>
       <c r="F399">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="G399" t="s">
         <v>38</v>
@@ -14305,7 +14305,7 @@
         <v>37</v>
       </c>
       <c r="F400">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="G400" t="s">
         <v>38</v>
@@ -14331,7 +14331,7 @@
         <v>37</v>
       </c>
       <c r="F401">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="G401" t="s">
         <v>38</v>
@@ -14357,7 +14357,7 @@
         <v>37</v>
       </c>
       <c r="F402">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="G402" t="s">
         <v>38</v>
@@ -14383,7 +14383,7 @@
         <v>37</v>
       </c>
       <c r="F403">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="G403" t="s">
         <v>38</v>
@@ -14409,7 +14409,7 @@
         <v>37</v>
       </c>
       <c r="F404">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="G404" t="s">
         <v>38</v>
@@ -14435,7 +14435,7 @@
         <v>37</v>
       </c>
       <c r="F405">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="G405" t="s">
         <v>38</v>
@@ -14461,7 +14461,7 @@
         <v>37</v>
       </c>
       <c r="F406">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G406" t="s">
         <v>38</v>
@@ -14487,7 +14487,7 @@
         <v>37</v>
       </c>
       <c r="F407">
-        <v>53</v>
+        <v>28</v>
       </c>
       <c r="G407" t="s">
         <v>38</v>
@@ -14513,7 +14513,7 @@
         <v>37</v>
       </c>
       <c r="F408">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G408" t="s">
         <v>38</v>
@@ -14539,7 +14539,7 @@
         <v>37</v>
       </c>
       <c r="F409">
-        <v>17</v>
+        <v>50</v>
       </c>
       <c r="G409" t="s">
         <v>38</v>
@@ -14565,7 +14565,7 @@
         <v>37</v>
       </c>
       <c r="F410">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="G410" t="s">
         <v>38</v>
@@ -14591,7 +14591,7 @@
         <v>37</v>
       </c>
       <c r="F411">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="G411" t="s">
         <v>38</v>
@@ -14617,7 +14617,7 @@
         <v>37</v>
       </c>
       <c r="F412">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="G412" t="s">
         <v>38</v>
@@ -14643,7 +14643,7 @@
         <v>37</v>
       </c>
       <c r="F413">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G413" t="s">
         <v>38</v>
@@ -14669,7 +14669,7 @@
         <v>37</v>
       </c>
       <c r="F414">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="G414" t="s">
         <v>38</v>
@@ -14695,7 +14695,7 @@
         <v>37</v>
       </c>
       <c r="F415">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="G415" t="s">
         <v>38</v>
@@ -14721,7 +14721,7 @@
         <v>37</v>
       </c>
       <c r="F416">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G416" t="s">
         <v>38</v>
@@ -14747,7 +14747,7 @@
         <v>37</v>
       </c>
       <c r="F417">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="G417" t="s">
         <v>38</v>
@@ -14773,7 +14773,7 @@
         <v>37</v>
       </c>
       <c r="F418">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G418" t="s">
         <v>38</v>
@@ -14799,7 +14799,7 @@
         <v>37</v>
       </c>
       <c r="F419">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="G419" t="s">
         <v>38</v>
@@ -14825,7 +14825,7 @@
         <v>37</v>
       </c>
       <c r="F420">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G420" t="s">
         <v>38</v>
@@ -14851,7 +14851,7 @@
         <v>37</v>
       </c>
       <c r="F421">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G421" t="s">
         <v>38</v>
@@ -14877,7 +14877,7 @@
         <v>37</v>
       </c>
       <c r="F422">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="G422" t="s">
         <v>38</v>
@@ -14903,7 +14903,7 @@
         <v>37</v>
       </c>
       <c r="F423">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G423" t="s">
         <v>38</v>
@@ -14929,7 +14929,7 @@
         <v>37</v>
       </c>
       <c r="F424">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G424" t="s">
         <v>38</v>
@@ -14955,7 +14955,7 @@
         <v>37</v>
       </c>
       <c r="F425">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="G425" t="s">
         <v>38</v>
@@ -14981,7 +14981,7 @@
         <v>37</v>
       </c>
       <c r="F426">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="G426" t="s">
         <v>38</v>
@@ -15007,7 +15007,7 @@
         <v>37</v>
       </c>
       <c r="F427">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="G427" t="s">
         <v>38</v>
@@ -15033,7 +15033,7 @@
         <v>37</v>
       </c>
       <c r="F428">
-        <v>35</v>
+        <v>47</v>
       </c>
       <c r="G428" t="s">
         <v>38</v>
@@ -15059,7 +15059,7 @@
         <v>37</v>
       </c>
       <c r="F429">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G429" t="s">
         <v>38</v>
@@ -15085,7 +15085,7 @@
         <v>37</v>
       </c>
       <c r="F430">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="G430" t="s">
         <v>38</v>
@@ -15111,7 +15111,7 @@
         <v>37</v>
       </c>
       <c r="F431">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="G431" t="s">
         <v>38</v>
@@ -15137,7 +15137,7 @@
         <v>37</v>
       </c>
       <c r="F432">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="G432" t="s">
         <v>38</v>
@@ -15163,7 +15163,7 @@
         <v>37</v>
       </c>
       <c r="F433">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G433" t="s">
         <v>38</v>
@@ -15189,7 +15189,7 @@
         <v>37</v>
       </c>
       <c r="F434">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="G434" t="s">
         <v>38</v>
@@ -15215,7 +15215,7 @@
         <v>37</v>
       </c>
       <c r="F435">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G435" t="s">
         <v>38</v>
@@ -15241,7 +15241,7 @@
         <v>37</v>
       </c>
       <c r="F436">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="G436" t="s">
         <v>38</v>
@@ -15267,7 +15267,7 @@
         <v>37</v>
       </c>
       <c r="F437">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G437" t="s">
         <v>38</v>
@@ -15293,7 +15293,7 @@
         <v>37</v>
       </c>
       <c r="F438">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="G438" t="s">
         <v>38</v>
@@ -15319,7 +15319,7 @@
         <v>37</v>
       </c>
       <c r="F439">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G439" t="s">
         <v>38</v>
@@ -15345,7 +15345,7 @@
         <v>37</v>
       </c>
       <c r="F440">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="G440" t="s">
         <v>38</v>
@@ -15371,7 +15371,7 @@
         <v>37</v>
       </c>
       <c r="F441">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="G441" t="s">
         <v>38</v>
@@ -15397,7 +15397,7 @@
         <v>37</v>
       </c>
       <c r="F442">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="G442" t="s">
         <v>38</v>
@@ -15423,7 +15423,7 @@
         <v>37</v>
       </c>
       <c r="F443">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G443" t="s">
         <v>38</v>
@@ -15449,7 +15449,7 @@
         <v>37</v>
       </c>
       <c r="F444">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G444" t="s">
         <v>38</v>
@@ -15475,7 +15475,7 @@
         <v>37</v>
       </c>
       <c r="F445">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="G445" t="s">
         <v>38</v>
@@ -15501,7 +15501,7 @@
         <v>37</v>
       </c>
       <c r="F446">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="G446" t="s">
         <v>38</v>
@@ -15527,7 +15527,7 @@
         <v>37</v>
       </c>
       <c r="F447">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="G447" t="s">
         <v>38</v>
@@ -15553,7 +15553,7 @@
         <v>37</v>
       </c>
       <c r="F448">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="G448" t="s">
         <v>38</v>
@@ -15579,7 +15579,7 @@
         <v>37</v>
       </c>
       <c r="F449">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G449" t="s">
         <v>38</v>
@@ -15605,7 +15605,7 @@
         <v>37</v>
       </c>
       <c r="F450">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G450" t="s">
         <v>38</v>
@@ -15631,7 +15631,7 @@
         <v>37</v>
       </c>
       <c r="F451">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="G451" t="s">
         <v>38</v>
@@ -15657,7 +15657,7 @@
         <v>37</v>
       </c>
       <c r="F452">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="G452" t="s">
         <v>38</v>
@@ -15683,7 +15683,7 @@
         <v>37</v>
       </c>
       <c r="F453">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="G453" t="s">
         <v>38</v>
@@ -15709,7 +15709,7 @@
         <v>37</v>
       </c>
       <c r="F454">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="G454" t="s">
         <v>38</v>
@@ -15735,7 +15735,7 @@
         <v>37</v>
       </c>
       <c r="F455">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="G455" t="s">
         <v>38</v>
@@ -15761,7 +15761,7 @@
         <v>37</v>
       </c>
       <c r="F456">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="G456" t="s">
         <v>38</v>
@@ -15787,7 +15787,7 @@
         <v>37</v>
       </c>
       <c r="F457">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G457" t="s">
         <v>38</v>
@@ -15813,7 +15813,7 @@
         <v>37</v>
       </c>
       <c r="F458">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="G458" t="s">
         <v>38</v>
@@ -15839,7 +15839,7 @@
         <v>37</v>
       </c>
       <c r="F459">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="G459" t="s">
         <v>38</v>
@@ -15865,7 +15865,7 @@
         <v>37</v>
       </c>
       <c r="F460">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="G460" t="s">
         <v>38</v>
@@ -15891,7 +15891,7 @@
         <v>37</v>
       </c>
       <c r="F461">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G461" t="s">
         <v>38</v>
@@ -15917,7 +15917,7 @@
         <v>37</v>
       </c>
       <c r="F462">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="G462" t="s">
         <v>38</v>
@@ -15943,7 +15943,7 @@
         <v>37</v>
       </c>
       <c r="F463">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G463" t="s">
         <v>38</v>
@@ -15969,7 +15969,7 @@
         <v>37</v>
       </c>
       <c r="F464">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G464" t="s">
         <v>38</v>
@@ -15995,7 +15995,7 @@
         <v>37</v>
       </c>
       <c r="F465">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G465" t="s">
         <v>38</v>
@@ -16021,7 +16021,7 @@
         <v>37</v>
       </c>
       <c r="F466">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="G466" t="s">
         <v>38</v>
@@ -16047,7 +16047,7 @@
         <v>37</v>
       </c>
       <c r="F467">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="G467" t="s">
         <v>38</v>
@@ -16073,7 +16073,7 @@
         <v>37</v>
       </c>
       <c r="F468">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="G468" t="s">
         <v>38</v>
@@ -16099,7 +16099,7 @@
         <v>37</v>
       </c>
       <c r="F469">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="G469" t="s">
         <v>38</v>
@@ -16125,7 +16125,7 @@
         <v>37</v>
       </c>
       <c r="F470">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="G470" t="s">
         <v>38</v>
@@ -16151,7 +16151,7 @@
         <v>37</v>
       </c>
       <c r="F471">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="G471" t="s">
         <v>38</v>
@@ -16177,7 +16177,7 @@
         <v>37</v>
       </c>
       <c r="F472">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="G472" t="s">
         <v>38</v>
@@ -16203,7 +16203,7 @@
         <v>37</v>
       </c>
       <c r="F473">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G473" t="s">
         <v>38</v>
@@ -16229,7 +16229,7 @@
         <v>37</v>
       </c>
       <c r="F474">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="G474" t="s">
         <v>38</v>
@@ -16255,7 +16255,7 @@
         <v>37</v>
       </c>
       <c r="F475">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="G475" t="s">
         <v>38</v>
@@ -16281,7 +16281,7 @@
         <v>37</v>
       </c>
       <c r="F476">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="G476" t="s">
         <v>38</v>
@@ -16307,7 +16307,7 @@
         <v>37</v>
       </c>
       <c r="F477">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="G477" t="s">
         <v>38</v>
@@ -16333,7 +16333,7 @@
         <v>37</v>
       </c>
       <c r="F478">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="G478" t="s">
         <v>38</v>
@@ -16359,7 +16359,7 @@
         <v>37</v>
       </c>
       <c r="F479">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="G479" t="s">
         <v>38</v>
@@ -16385,7 +16385,7 @@
         <v>37</v>
       </c>
       <c r="F480">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="G480" t="s">
         <v>38</v>
@@ -16411,7 +16411,7 @@
         <v>37</v>
       </c>
       <c r="F481">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G481" t="s">
         <v>38</v>
@@ -16437,7 +16437,7 @@
         <v>37</v>
       </c>
       <c r="F482">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="G482" t="s">
         <v>38</v>
@@ -16463,7 +16463,7 @@
         <v>37</v>
       </c>
       <c r="F483">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G483" t="s">
         <v>38</v>
@@ -16489,7 +16489,7 @@
         <v>37</v>
       </c>
       <c r="F484">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G484" t="s">
         <v>38</v>
@@ -16541,7 +16541,7 @@
         <v>37</v>
       </c>
       <c r="F486">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="G486" t="s">
         <v>38</v>
@@ -16567,7 +16567,7 @@
         <v>37</v>
       </c>
       <c r="F487">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="G487" t="s">
         <v>38</v>
@@ -16593,7 +16593,7 @@
         <v>37</v>
       </c>
       <c r="F488">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="G488" t="s">
         <v>38</v>
@@ -16619,7 +16619,7 @@
         <v>37</v>
       </c>
       <c r="F489">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="G489" t="s">
         <v>38</v>
@@ -16645,7 +16645,7 @@
         <v>37</v>
       </c>
       <c r="F490">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="G490" t="s">
         <v>38</v>
@@ -16671,7 +16671,7 @@
         <v>37</v>
       </c>
       <c r="F491">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G491" t="s">
         <v>38</v>
@@ -16697,7 +16697,7 @@
         <v>37</v>
       </c>
       <c r="F492">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="G492" t="s">
         <v>38</v>
@@ -16723,7 +16723,7 @@
         <v>37</v>
       </c>
       <c r="F493">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="G493" t="s">
         <v>38</v>
@@ -16749,7 +16749,7 @@
         <v>37</v>
       </c>
       <c r="F494">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G494" t="s">
         <v>38</v>
@@ -16775,7 +16775,7 @@
         <v>37</v>
       </c>
       <c r="F495">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G495" t="s">
         <v>38</v>
@@ -16801,7 +16801,7 @@
         <v>37</v>
       </c>
       <c r="F496">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="G496" t="s">
         <v>38</v>
@@ -16827,7 +16827,7 @@
         <v>37</v>
       </c>
       <c r="F497">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="G497" t="s">
         <v>38</v>
@@ -16853,7 +16853,7 @@
         <v>37</v>
       </c>
       <c r="F498">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G498" t="s">
         <v>38</v>
@@ -16879,7 +16879,7 @@
         <v>37</v>
       </c>
       <c r="F499">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="G499" t="s">
         <v>38</v>
@@ -16905,7 +16905,7 @@
         <v>37</v>
       </c>
       <c r="F500">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="G500" t="s">
         <v>38</v>
@@ -16931,7 +16931,7 @@
         <v>37</v>
       </c>
       <c r="F501">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="G501" t="s">
         <v>38</v>

</xml_diff>